<commit_message>
updated node_metrix_150/200 with the pipeline connections of node_metrics
</commit_message>
<xml_diff>
--- a/southern_europe/italy_data/geographical_feature/node_metrics.xlsx
+++ b/southern_europe/italy_data/geographical_feature/node_metrics.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\0954659\PycharmProjects\AdOpT-NET0_luca\southern_europe\italy_data\geographical_feature\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{14CDD1E0-BF5A-4A58-884A-09C7D9882B7A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8F0B1B6C-90B1-4D3F-94DE-5932F283F62D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-75" yWindow="-16320" windowWidth="29040" windowHeight="15720" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="38304" yWindow="-4260" windowWidth="15552" windowHeight="16656" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="nodes" sheetId="1" r:id="rId1"/>
@@ -19145,958 +19145,958 @@
     <row r="46" spans="1:45" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
     <row r="47" spans="1:45" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
     <row r="48" spans="1:45" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="49" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="50" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="51" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="52" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="53" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="54" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="55" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="56" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="57" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="58" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="59" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="60" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="61" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="62" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="63" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="64" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="65" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="66" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="67" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="68" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="69" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="70" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="71" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="72" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="73" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="74" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="75" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="76" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="77" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="78" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="79" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="80" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="81" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="82" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="83" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="84" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="85" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="86" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="87" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="88" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="89" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="90" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="91" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="92" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="93" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="94" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="95" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="96" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="97" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="98" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="99" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="100" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="101" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="102" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="103" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="104" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="105" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="106" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="107" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="108" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="109" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="110" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="111" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="112" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="113" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="114" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="115" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="116" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="117" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="118" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="119" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="120" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="121" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="122" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="123" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="124" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="125" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="126" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="127" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="128" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="129" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="130" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="131" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="132" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="133" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="134" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="135" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="136" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="137" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="138" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="139" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="140" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="141" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="142" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="143" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="144" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="145" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="146" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="147" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="148" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="149" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="150" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="151" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="152" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="153" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="154" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="155" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="156" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="157" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="158" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="159" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="160" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="161" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="162" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="163" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="164" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="165" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="166" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="167" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="168" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="169" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="170" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="171" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="172" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="173" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="174" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="175" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="176" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="177" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="178" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="179" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="180" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="181" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="182" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="183" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="184" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="185" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="186" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="187" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="188" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="189" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="190" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="191" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="192" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="193" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="194" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="195" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="196" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="197" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="198" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="199" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="200" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="201" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="202" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="203" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="204" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="205" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="206" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="207" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="208" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="209" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="210" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="211" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="212" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="213" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="214" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="215" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="216" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="217" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="218" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="219" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="220" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="221" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="222" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="223" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="224" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="225" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="226" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="227" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="228" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="229" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="230" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="231" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="232" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="233" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="234" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="235" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="236" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="237" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="238" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="239" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="240" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="241" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="242" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="243" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="244" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="245" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="246" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="247" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="248" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="249" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="250" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="251" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="252" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="253" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="254" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="255" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="256" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="257" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="258" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="259" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="260" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="261" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="262" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="263" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="264" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="265" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="266" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="267" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="268" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="269" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="270" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="271" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="272" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="273" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="274" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="275" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="276" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="277" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="278" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="279" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="280" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="281" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="282" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="283" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="284" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="285" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="286" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="287" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="288" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="289" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="290" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="291" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="292" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="293" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="294" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="295" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="296" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="297" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="298" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="299" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="300" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="301" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="302" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="303" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="304" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="305" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="306" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="307" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="308" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="309" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="310" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="311" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="312" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="313" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="314" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="315" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="316" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="317" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="318" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="319" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="320" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="321" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="322" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="323" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="324" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="325" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="326" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="327" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="328" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="329" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="330" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="331" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="332" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="333" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="334" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="335" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="336" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="337" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="338" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="339" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="340" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="341" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="342" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="343" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="344" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="345" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="346" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="347" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="348" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="349" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="350" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="351" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="352" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="353" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="354" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="355" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="356" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="357" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="358" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="359" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="360" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="361" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="362" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="363" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="364" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="365" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="366" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="367" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="368" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="369" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="370" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="371" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="372" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="373" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="374" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="375" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="376" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="377" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="378" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="379" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="380" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="381" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="382" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="383" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="384" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="385" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="386" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="387" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="388" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="389" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="390" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="391" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="392" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="393" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="394" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="395" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="396" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="397" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="398" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="399" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="400" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="401" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="402" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="403" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="404" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="405" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="406" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="407" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="408" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="409" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="410" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="411" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="412" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="413" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="414" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="415" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="416" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="417" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="418" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="419" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="420" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="421" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="422" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="423" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="424" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="425" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="426" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="427" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="428" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="429" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="430" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="431" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="432" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="433" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="434" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="435" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="436" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="437" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="438" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="439" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="440" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="441" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="442" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="443" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="444" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="445" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="446" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="447" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="448" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="449" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="450" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="451" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="452" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="453" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="454" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="455" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="456" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="457" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="458" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="459" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="460" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="461" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="462" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="463" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="464" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="465" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="466" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="467" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="468" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="469" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="470" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="471" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="472" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="473" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="474" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="475" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="476" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="477" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="478" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="479" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="480" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="481" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="482" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="483" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="484" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="485" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="486" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="487" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="488" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="489" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="490" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="491" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="492" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="493" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="494" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="495" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="496" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="497" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="498" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="499" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="500" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="501" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="502" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="503" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="504" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="505" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="506" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="507" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="508" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="509" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="510" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="511" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="512" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="513" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="514" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="515" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="516" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="517" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="518" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="519" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="520" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="521" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="522" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="523" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="524" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="525" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="526" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="527" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="528" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="529" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="530" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="531" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="532" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="533" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="534" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="535" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="536" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="537" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="538" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="539" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="540" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="541" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="542" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="543" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="544" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="545" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="546" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="547" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="548" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="549" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="550" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="551" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="552" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="553" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="554" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="555" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="556" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="557" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="558" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="559" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="560" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="561" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="562" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="563" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="564" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="565" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="566" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="567" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="568" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="569" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="570" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="571" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="572" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="573" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="574" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="575" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="576" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="577" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="578" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="579" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="580" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="581" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="582" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="583" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="584" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="585" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="586" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="587" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="588" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="589" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="590" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="591" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="592" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="593" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="594" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="595" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="596" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="597" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="598" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="599" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="600" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="601" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="602" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="603" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="604" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="605" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="606" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="607" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="608" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="609" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="610" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="611" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="612" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="613" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="614" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="615" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="616" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="617" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="618" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="619" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="620" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="621" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="622" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="623" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="624" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="625" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="626" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="627" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="628" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="629" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="630" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="631" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="632" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="633" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="634" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="635" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="636" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="637" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="638" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="639" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="640" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="641" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="642" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="643" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="644" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="645" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="646" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="647" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="648" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="649" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="650" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="651" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="652" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="653" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="654" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="655" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="656" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="657" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="658" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="659" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="660" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="661" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="662" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="663" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="664" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="665" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="666" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="667" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="668" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="669" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="670" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="671" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="672" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="673" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="674" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="675" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="676" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="677" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="678" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="679" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="680" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="681" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="682" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="683" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="684" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="685" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="686" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="687" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="688" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="689" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="690" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="691" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="692" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="693" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="694" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="695" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="696" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="697" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="698" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="699" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="700" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="701" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="702" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="703" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="704" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="705" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="706" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="707" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="708" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="709" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="710" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="711" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="712" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="713" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="714" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="715" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="716" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="717" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="718" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="719" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="720" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="721" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="722" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="723" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="724" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="725" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="726" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="727" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="728" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="729" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="730" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="731" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="732" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="733" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="734" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="735" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="736" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="737" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="738" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="739" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="740" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="741" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="742" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="743" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="744" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="745" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="746" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="747" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="748" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="749" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="750" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="751" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="752" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="753" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="754" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="755" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="756" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="757" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="758" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="759" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="760" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="761" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="762" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="763" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="764" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="765" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="766" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="767" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="768" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="769" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="770" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="771" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="772" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="773" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="774" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="775" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="776" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="777" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="778" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="779" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="780" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="781" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="782" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="783" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="784" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="785" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="786" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="787" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="788" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="789" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="790" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="791" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="792" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="793" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="794" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="795" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="796" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="797" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="798" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="799" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="800" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="801" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="802" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="803" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="804" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="805" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="806" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="807" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="808" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="809" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="810" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="811" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="812" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="813" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="814" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="815" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="816" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="817" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="818" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="819" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="820" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="821" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="822" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="823" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="824" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="825" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="826" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="827" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="828" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="829" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="830" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="831" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="832" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="833" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="834" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="835" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="836" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="837" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="838" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="839" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="840" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="841" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="842" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="843" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="844" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="845" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="846" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="847" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="848" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="849" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="850" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="851" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="852" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="853" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="854" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="855" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="856" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="857" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="858" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="859" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="860" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="861" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="862" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="863" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="864" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="865" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="866" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="867" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="868" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="869" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="870" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="871" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="872" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="873" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="874" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="875" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="876" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="877" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="878" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="879" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="880" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="881" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="882" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="883" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="884" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="885" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="886" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="887" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="888" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="889" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="890" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="891" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="892" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="893" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="894" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="895" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="896" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="897" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="898" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="899" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="900" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="901" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="902" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="903" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="904" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="905" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="906" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="907" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="908" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="909" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="910" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="911" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="912" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="913" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="914" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="915" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="916" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="917" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="918" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="919" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="920" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="921" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="922" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="923" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="924" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="925" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="926" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="927" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="928" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="929" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="930" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="931" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="932" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="933" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="934" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="935" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="936" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="937" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="938" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="939" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="940" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="941" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="942" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="943" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="944" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="945" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="946" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="947" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="948" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="949" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="950" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="951" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="952" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="953" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="954" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="955" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="956" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="957" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="958" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="959" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="960" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="961" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="962" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="963" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="964" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="965" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="966" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="967" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="968" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="969" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="970" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="971" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="972" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="973" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="974" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="975" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="976" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="977" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="978" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="979" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="980" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="981" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="982" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="983" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="984" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="985" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="986" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="987" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="988" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="989" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="990" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="991" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="992" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="993" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="994" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="995" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="996" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="997" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="998" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="999" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="1000" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="49" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="50" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="51" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="52" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="53" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="54" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="55" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="56" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="57" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="58" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="59" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="60" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="61" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="62" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="63" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="64" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="65" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="66" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="67" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="68" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="69" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="70" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="71" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="72" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="73" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="74" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="75" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="76" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="77" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="78" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="79" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="80" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="81" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="82" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="83" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="84" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="85" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="86" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="87" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="88" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="89" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="90" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="91" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="92" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="93" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="94" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="95" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="96" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="97" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="98" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="99" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="100" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="101" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="102" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="103" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="104" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="105" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="106" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="107" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="108" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="109" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="110" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="111" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="112" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="113" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="114" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="115" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="116" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="117" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="118" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="119" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="120" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="121" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="122" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="123" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="124" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="125" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="126" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="127" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="128" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="129" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="130" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="131" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="132" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="133" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="134" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="135" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="136" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="137" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="138" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="139" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="140" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="141" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="142" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="143" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="144" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="145" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="146" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="147" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="148" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="149" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="150" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="151" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="152" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="153" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="154" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="155" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="156" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="157" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="158" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="159" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="160" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="161" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="162" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="163" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="164" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="165" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="166" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="167" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="168" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="169" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="170" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="171" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="172" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="173" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="174" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="175" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="176" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="177" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="178" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="179" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="180" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="181" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="182" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="183" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="184" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="185" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="186" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="187" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="188" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="189" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="190" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="191" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="192" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="193" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="194" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="195" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="196" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="197" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="198" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="199" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="200" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="201" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="202" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="203" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="204" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="205" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="206" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="207" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="208" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="209" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="210" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="211" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="212" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="213" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="214" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="215" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="216" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="217" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="218" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="219" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="220" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="221" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="222" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="223" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="224" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="225" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="226" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="227" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="228" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="229" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="230" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="231" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="232" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="233" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="234" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="235" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="236" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="237" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="238" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="239" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="240" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="241" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="242" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="243" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="244" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="245" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="246" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="247" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="248" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="249" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="250" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="251" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="252" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="253" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="254" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="255" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="256" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="257" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="258" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="259" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="260" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="261" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="262" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="263" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="264" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="265" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="266" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="267" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="268" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="269" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="270" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="271" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="272" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="273" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="274" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="275" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="276" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="277" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="278" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="279" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="280" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="281" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="282" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="283" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="284" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="285" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="286" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="287" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="288" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="289" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="290" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="291" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="292" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="293" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="294" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="295" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="296" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="297" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="298" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="299" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="300" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="301" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="302" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="303" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="304" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="305" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="306" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="307" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="308" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="309" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="310" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="311" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="312" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="313" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="314" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="315" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="316" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="317" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="318" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="319" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="320" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="321" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="322" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="323" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="324" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="325" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="326" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="327" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="328" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="329" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="330" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="331" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="332" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="333" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="334" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="335" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="336" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="337" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="338" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="339" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="340" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="341" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="342" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="343" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="344" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="345" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="346" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="347" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="348" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="349" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="350" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="351" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="352" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="353" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="354" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="355" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="356" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="357" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="358" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="359" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="360" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="361" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="362" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="363" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="364" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="365" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="366" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="367" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="368" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="369" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="370" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="371" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="372" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="373" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="374" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="375" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="376" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="377" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="378" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="379" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="380" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="381" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="382" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="383" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="384" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="385" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="386" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="387" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="388" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="389" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="390" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="391" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="392" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="393" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="394" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="395" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="396" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="397" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="398" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="399" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="400" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="401" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="402" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="403" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="404" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="405" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="406" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="407" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="408" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="409" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="410" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="411" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="412" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="413" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="414" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="415" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="416" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="417" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="418" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="419" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="420" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="421" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="422" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="423" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="424" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="425" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="426" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="427" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="428" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="429" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="430" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="431" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="432" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="433" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="434" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="435" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="436" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="437" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="438" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="439" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="440" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="441" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="442" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="443" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="444" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="445" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="446" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="447" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="448" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="449" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="450" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="451" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="452" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="453" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="454" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="455" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="456" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="457" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="458" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="459" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="460" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="461" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="462" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="463" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="464" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="465" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="466" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="467" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="468" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="469" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="470" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="471" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="472" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="473" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="474" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="475" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="476" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="477" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="478" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="479" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="480" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="481" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="482" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="483" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="484" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="485" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="486" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="487" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="488" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="489" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="490" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="491" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="492" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="493" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="494" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="495" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="496" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="497" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="498" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="499" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="500" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="501" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="502" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="503" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="504" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="505" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="506" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="507" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="508" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="509" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="510" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="511" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="512" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="513" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="514" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="515" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="516" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="517" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="518" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="519" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="520" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="521" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="522" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="523" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="524" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="525" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="526" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="527" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="528" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="529" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="530" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="531" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="532" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="533" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="534" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="535" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="536" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="537" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="538" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="539" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="540" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="541" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="542" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="543" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="544" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="545" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="546" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="547" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="548" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="549" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="550" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="551" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="552" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="553" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="554" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="555" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="556" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="557" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="558" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="559" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="560" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="561" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="562" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="563" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="564" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="565" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="566" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="567" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="568" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="569" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="570" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="571" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="572" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="573" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="574" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="575" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="576" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="577" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="578" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="579" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="580" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="581" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="582" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="583" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="584" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="585" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="586" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="587" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="588" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="589" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="590" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="591" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="592" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="593" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="594" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="595" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="596" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="597" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="598" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="599" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="600" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="601" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="602" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="603" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="604" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="605" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="606" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="607" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="608" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="609" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="610" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="611" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="612" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="613" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="614" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="615" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="616" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="617" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="618" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="619" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="620" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="621" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="622" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="623" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="624" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="625" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="626" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="627" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="628" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="629" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="630" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="631" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="632" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="633" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="634" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="635" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="636" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="637" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="638" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="639" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="640" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="641" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="642" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="643" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="644" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="645" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="646" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="647" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="648" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="649" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="650" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="651" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="652" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="653" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="654" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="655" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="656" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="657" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="658" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="659" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="660" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="661" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="662" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="663" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="664" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="665" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="666" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="667" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="668" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="669" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="670" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="671" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="672" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="673" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="674" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="675" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="676" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="677" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="678" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="679" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="680" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="681" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="682" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="683" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="684" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="685" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="686" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="687" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="688" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="689" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="690" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="691" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="692" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="693" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="694" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="695" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="696" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="697" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="698" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="699" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="700" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="701" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="702" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="703" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="704" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="705" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="706" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="707" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="708" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="709" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="710" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="711" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="712" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="713" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="714" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="715" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="716" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="717" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="718" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="719" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="720" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="721" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="722" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="723" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="724" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="725" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="726" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="727" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="728" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="729" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="730" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="731" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="732" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="733" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="734" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="735" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="736" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="737" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="738" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="739" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="740" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="741" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="742" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="743" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="744" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="745" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="746" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="747" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="748" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="749" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="750" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="751" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="752" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="753" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="754" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="755" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="756" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="757" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="758" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="759" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="760" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="761" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="762" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="763" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="764" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="765" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="766" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="767" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="768" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="769" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="770" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="771" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="772" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="773" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="774" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="775" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="776" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="777" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="778" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="779" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="780" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="781" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="782" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="783" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="784" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="785" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="786" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="787" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="788" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="789" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="790" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="791" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="792" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="793" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="794" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="795" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="796" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="797" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="798" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="799" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="800" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="801" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="802" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="803" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="804" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="805" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="806" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="807" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="808" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="809" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="810" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="811" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="812" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="813" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="814" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="815" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="816" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="817" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="818" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="819" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="820" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="821" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="822" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="823" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="824" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="825" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="826" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="827" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="828" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="829" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="830" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="831" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="832" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="833" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="834" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="835" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="836" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="837" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="838" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="839" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="840" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="841" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="842" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="843" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="844" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="845" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="846" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="847" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="848" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="849" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="850" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="851" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="852" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="853" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="854" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="855" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="856" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="857" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="858" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="859" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="860" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="861" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="862" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="863" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="864" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="865" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="866" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="867" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="868" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="869" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="870" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="871" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="872" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="873" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="874" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="875" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="876" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="877" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="878" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="879" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="880" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="881" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="882" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="883" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="884" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="885" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="886" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="887" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="888" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="889" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="890" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="891" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="892" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="893" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="894" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="895" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="896" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="897" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="898" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="899" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="900" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="901" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="902" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="903" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="904" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="905" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="906" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="907" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="908" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="909" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="910" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="911" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="912" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="913" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="914" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="915" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="916" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="917" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="918" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="919" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="920" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="921" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="922" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="923" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="924" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="925" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="926" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="927" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="928" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="929" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="930" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="931" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="932" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="933" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="934" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="935" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="936" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="937" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="938" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="939" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="940" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="941" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="942" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="943" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="944" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="945" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="946" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="947" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="948" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="949" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="950" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="951" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="952" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="953" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="954" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="955" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="956" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="957" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="958" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="959" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="960" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="961" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="962" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="963" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="964" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="965" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="966" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="967" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="968" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="969" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="970" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="971" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="972" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="973" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="974" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="975" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="976" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="977" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="978" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="979" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="980" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="981" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="982" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="983" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="984" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="985" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="986" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="987" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="988" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="989" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="990" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="991" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="992" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="993" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="994" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="995" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="996" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="997" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="998" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="999" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="1000" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
   </sheetData>
   <conditionalFormatting sqref="B2:Y45 Z2:AB44 AC2:AC45 AD2:AD44 AE2:AS45">
     <cfRule type="colorScale" priority="3">

</xml_diff>

<commit_message>
fixed opex_var_arc naming with semicolumn
</commit_message>
<xml_diff>
--- a/southern_europe/italy_data/geographical_feature/node_metrics.xlsx
+++ b/southern_europe/italy_data/geographical_feature/node_metrics.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\0954659\PycharmProjects\AdOpT-NET0_luca\southern_europe\italy_data\geographical_feature\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8F0B1B6C-90B1-4D3F-94DE-5932F283F62D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2B3C1B2B-48C0-4613-8342-018C8D2C2E2B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="38304" yWindow="-4260" windowWidth="15552" windowHeight="16656" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="22932" yWindow="-4368" windowWidth="30936" windowHeight="16776" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="nodes" sheetId="1" r:id="rId1"/>
@@ -141,9 +141,6 @@
   </si>
   <si>
     <t>Termovalorizzatore di Dalmine</t>
-  </si>
-  <si>
-    <t>Piacenza</t>
   </si>
   <si>
     <t>VERNASCA cement plant</t>
@@ -537,6 +534,9 @@
   </si>
   <si>
     <t>Hypothetical potential transport switch</t>
+  </si>
+  <si>
+    <t>Piacenza</t>
   </si>
 </sst>
 </file>
@@ -1417,7 +1417,7 @@
         <v>20</v>
       </c>
       <c r="B21" s="21" t="s">
-        <v>31</v>
+        <v>162</v>
       </c>
       <c r="C21" s="2">
         <v>9.7038200000000003</v>
@@ -1444,7 +1444,7 @@
         <v>20</v>
       </c>
       <c r="B22" s="21" t="s">
-        <v>31</v>
+        <v>162</v>
       </c>
       <c r="C22" s="2">
         <v>9.7038200000000003</v>
@@ -1468,7 +1468,7 @@
         <v>21</v>
       </c>
       <c r="B23" s="21" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="C23" s="2">
         <v>9.8099799999999995</v>
@@ -1495,7 +1495,7 @@
         <v>22</v>
       </c>
       <c r="B24" s="21" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="C24" s="2">
         <v>10.047169999999999</v>
@@ -1518,7 +1518,7 @@
         <v>23</v>
       </c>
       <c r="B25" s="21" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="C25" s="2">
         <v>10.20872</v>
@@ -1541,7 +1541,7 @@
         <v>24</v>
       </c>
       <c r="B26" s="21" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="C26" s="2">
         <v>10.341900000000001</v>
@@ -1564,7 +1564,7 @@
         <v>25</v>
       </c>
       <c r="B27" s="21" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="C27" s="2">
         <v>10.35805</v>
@@ -1590,7 +1590,7 @@
         <v>26</v>
       </c>
       <c r="B28" s="21" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="C28" s="2">
         <v>11.053699999999999</v>
@@ -1613,7 +1613,7 @@
         <v>27</v>
       </c>
       <c r="B29" s="21" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="C29" s="2">
         <v>10.943759999999999</v>
@@ -1636,7 +1636,7 @@
         <v>28</v>
       </c>
       <c r="B30" s="21" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="C30" s="2">
         <v>11.30925</v>
@@ -1659,7 +1659,7 @@
         <v>29</v>
       </c>
       <c r="B31" s="21" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="C31" s="2">
         <v>11.556369999999999</v>
@@ -1682,7 +1682,7 @@
         <v>30</v>
       </c>
       <c r="B32" s="21" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="C32" s="2">
         <v>11.428890000000001</v>
@@ -1705,7 +1705,7 @@
         <v>31</v>
       </c>
       <c r="B33" s="21" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="C33" s="2">
         <v>11.75079</v>
@@ -1731,7 +1731,7 @@
         <v>32</v>
       </c>
       <c r="B34" s="21" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="C34" s="5">
         <v>11.69642</v>
@@ -1754,7 +1754,7 @@
         <v>33</v>
       </c>
       <c r="B35" s="21" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="C35" s="2">
         <v>11.963570000000001</v>
@@ -1777,7 +1777,7 @@
         <v>34</v>
       </c>
       <c r="B36" s="21" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="C36" s="2">
         <v>11.924099999999999</v>
@@ -1800,7 +1800,7 @@
         <v>35</v>
       </c>
       <c r="B37" s="21" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="C37" s="2">
         <v>12.08798</v>
@@ -1823,7 +1823,7 @@
         <v>36</v>
       </c>
       <c r="B38" s="21" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="C38" s="2">
         <v>12.269209999999999</v>
@@ -1846,7 +1846,7 @@
         <v>37</v>
       </c>
       <c r="B39" s="21" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="C39" s="2">
         <v>12.2</v>
@@ -1862,7 +1862,7 @@
       </c>
       <c r="G39" s="3"/>
       <c r="H39" s="1" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
     </row>
     <row r="40" spans="1:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
@@ -1870,7 +1870,7 @@
         <v>38</v>
       </c>
       <c r="B40" s="21" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="C40" s="5">
         <v>12.31551</v>
@@ -1893,7 +1893,7 @@
         <v>39</v>
       </c>
       <c r="B41" s="21" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="C41" s="2">
         <v>12.74245</v>
@@ -1919,7 +1919,7 @@
         <v>40</v>
       </c>
       <c r="B42" s="21" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="C42" s="2">
         <v>12.63189</v>
@@ -1942,7 +1942,7 @@
         <v>41</v>
       </c>
       <c r="B43" s="21" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="C43" s="2">
         <v>13.80006</v>
@@ -1965,7 +1965,7 @@
         <v>42</v>
       </c>
       <c r="B44" s="21" t="s">
-        <v>161</v>
+        <v>160</v>
       </c>
       <c r="C44" s="2">
         <v>12.274480000000001</v>
@@ -1989,7 +1989,7 @@
         <v>43</v>
       </c>
       <c r="B45" s="21" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="C45" s="5">
         <v>12.564</v>
@@ -2005,7 +2005,7 @@
       </c>
       <c r="G45" s="7"/>
       <c r="H45" s="1" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
     </row>
     <row r="46" spans="1:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
@@ -2013,7 +2013,7 @@
         <v>44</v>
       </c>
       <c r="B46" s="4" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="C46" s="4">
         <v>10.64</v>
@@ -27287,45 +27287,45 @@
   <sheetData>
     <row r="1" spans="1:26" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A1" s="12" t="s">
+        <v>56</v>
+      </c>
+      <c r="B1" s="13" t="s">
         <v>57</v>
       </c>
-      <c r="B1" s="13" t="s">
+      <c r="C1" s="13" t="s">
         <v>58</v>
       </c>
-      <c r="C1" s="13" t="s">
+      <c r="D1" s="12" t="s">
         <v>59</v>
       </c>
-      <c r="D1" s="12" t="s">
+      <c r="E1" s="12" t="s">
         <v>60</v>
       </c>
-      <c r="E1" s="12" t="s">
+      <c r="F1" s="12" t="s">
         <v>61</v>
       </c>
-      <c r="F1" s="12" t="s">
+      <c r="G1" s="12" t="s">
         <v>62</v>
       </c>
-      <c r="G1" s="12" t="s">
+      <c r="H1" s="12" t="s">
         <v>63</v>
       </c>
-      <c r="H1" s="12" t="s">
+      <c r="I1" s="12" t="s">
         <v>64</v>
       </c>
-      <c r="I1" s="12" t="s">
+      <c r="J1" s="12" t="s">
         <v>65</v>
       </c>
-      <c r="J1" s="12" t="s">
+      <c r="K1" s="12" t="s">
         <v>66</v>
       </c>
-      <c r="K1" s="12" t="s">
+      <c r="L1" s="12" t="s">
         <v>67</v>
-      </c>
-      <c r="L1" s="12" t="s">
-        <v>68</v>
       </c>
     </row>
     <row r="2" spans="1:26" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A2" s="14" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="B2" s="15">
         <v>11.75079</v>
@@ -27340,25 +27340,25 @@
         <v>11</v>
       </c>
       <c r="F2" s="14" t="s">
+        <v>68</v>
+      </c>
+      <c r="G2" s="14" t="s">
         <v>69</v>
       </c>
-      <c r="G2" s="14" t="s">
+      <c r="H2" s="14" t="s">
         <v>70</v>
-      </c>
-      <c r="H2" s="14" t="s">
-        <v>71</v>
       </c>
       <c r="I2" s="14">
         <v>800000</v>
       </c>
       <c r="J2" s="14" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="K2" s="14">
         <v>2021</v>
       </c>
       <c r="L2" s="17" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="M2" s="18"/>
       <c r="N2" s="18"/>
@@ -27377,7 +27377,7 @@
     </row>
     <row r="3" spans="1:26" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A3" s="14" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="B3" s="15">
         <v>11.963570000000001</v>
@@ -27392,13 +27392,13 @@
         <v>11</v>
       </c>
       <c r="F3" s="14" t="s">
+        <v>73</v>
+      </c>
+      <c r="G3" s="14" t="s">
         <v>74</v>
       </c>
-      <c r="G3" s="14" t="s">
+      <c r="H3" s="14" t="s">
         <v>75</v>
-      </c>
-      <c r="H3" s="14" t="s">
-        <v>76</v>
       </c>
       <c r="I3" s="14">
         <v>1000000</v>
@@ -27408,7 +27408,7 @@
         <v>2021</v>
       </c>
       <c r="L3" s="17" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="M3" s="18"/>
       <c r="N3" s="18"/>
@@ -27427,7 +27427,7 @@
     </row>
     <row r="4" spans="1:26" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A4" s="14" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="B4" s="15">
         <v>12.269209999999999</v>
@@ -27442,23 +27442,23 @@
         <v>11</v>
       </c>
       <c r="F4" s="14" t="s">
+        <v>76</v>
+      </c>
+      <c r="G4" s="14" t="s">
+        <v>74</v>
+      </c>
+      <c r="H4" s="14" t="s">
         <v>77</v>
       </c>
-      <c r="G4" s="14" t="s">
-        <v>75</v>
-      </c>
-      <c r="H4" s="14" t="s">
+      <c r="I4" s="14" t="s">
         <v>78</v>
-      </c>
-      <c r="I4" s="14" t="s">
-        <v>79</v>
       </c>
       <c r="J4" s="14"/>
       <c r="K4" s="14">
         <v>2021</v>
       </c>
       <c r="L4" s="17" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="M4" s="18"/>
       <c r="N4" s="18"/>
@@ -27492,25 +27492,25 @@
         <v>11</v>
       </c>
       <c r="F5" s="14" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="G5" s="14" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="H5" s="14" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="I5" s="14">
         <v>1600000</v>
       </c>
       <c r="J5" s="14" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="K5" s="14">
         <v>2021</v>
       </c>
       <c r="L5" s="17" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="M5" s="18"/>
       <c r="N5" s="18"/>
@@ -27529,7 +27529,7 @@
     </row>
     <row r="6" spans="1:26" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A6" s="14" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="B6" s="15">
         <v>10.047129999999999</v>
@@ -27544,13 +27544,13 @@
         <v>11</v>
       </c>
       <c r="F6" s="14" t="s">
+        <v>80</v>
+      </c>
+      <c r="G6" s="14" t="s">
         <v>81</v>
       </c>
-      <c r="G6" s="14" t="s">
+      <c r="H6" s="14" t="s">
         <v>82</v>
-      </c>
-      <c r="H6" s="14" t="s">
-        <v>83</v>
       </c>
       <c r="I6" s="14"/>
       <c r="J6" s="14"/>
@@ -27558,7 +27558,7 @@
         <v>2021</v>
       </c>
       <c r="L6" s="17" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="M6" s="18"/>
       <c r="N6" s="18"/>
@@ -27592,25 +27592,25 @@
         <v>11</v>
       </c>
       <c r="F7" s="14" t="s">
+        <v>83</v>
+      </c>
+      <c r="G7" s="14" t="s">
+        <v>74</v>
+      </c>
+      <c r="H7" s="14" t="s">
         <v>84</v>
-      </c>
-      <c r="G7" s="14" t="s">
-        <v>75</v>
-      </c>
-      <c r="H7" s="14" t="s">
-        <v>85</v>
       </c>
       <c r="I7" s="14">
         <v>1500000</v>
       </c>
       <c r="J7" s="14" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="K7" s="14">
         <v>2021</v>
       </c>
       <c r="L7" s="17" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="M7" s="18"/>
       <c r="N7" s="18"/>
@@ -27644,21 +27644,21 @@
         <v>11</v>
       </c>
       <c r="F8" s="14" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="G8" s="14"/>
       <c r="H8" s="14" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="I8" s="14" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="J8" s="14"/>
       <c r="K8" s="14">
         <v>2021</v>
       </c>
       <c r="L8" s="17" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="M8" s="18"/>
       <c r="N8" s="18"/>
@@ -27677,7 +27677,7 @@
     </row>
     <row r="9" spans="1:26" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A9" s="14" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="B9" s="15">
         <v>10.341900000000001</v>
@@ -27692,25 +27692,25 @@
         <v>11</v>
       </c>
       <c r="F9" s="14" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="G9" s="14" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="H9" s="14" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="I9" s="14">
         <v>1300000</v>
       </c>
       <c r="J9" s="14" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="K9" s="14">
         <v>2021</v>
       </c>
       <c r="L9" s="17" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="M9" s="18"/>
       <c r="N9" s="18"/>
@@ -27729,7 +27729,7 @@
     </row>
     <row r="10" spans="1:26" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A10" s="14" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="B10" s="15">
         <v>10.047169999999999</v>
@@ -27744,23 +27744,23 @@
         <v>11</v>
       </c>
       <c r="F10" s="14" t="s">
+        <v>88</v>
+      </c>
+      <c r="G10" s="14" t="s">
+        <v>74</v>
+      </c>
+      <c r="H10" s="14" t="s">
         <v>89</v>
       </c>
-      <c r="G10" s="14" t="s">
-        <v>75</v>
-      </c>
-      <c r="H10" s="14" t="s">
-        <v>90</v>
-      </c>
       <c r="I10" s="14" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="J10" s="14"/>
       <c r="K10" s="14">
         <v>2021</v>
       </c>
       <c r="L10" s="17" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="M10" s="18"/>
       <c r="N10" s="18"/>
@@ -27794,23 +27794,23 @@
         <v>11</v>
       </c>
       <c r="F11" s="14" t="s">
+        <v>90</v>
+      </c>
+      <c r="G11" s="14" t="s">
+        <v>74</v>
+      </c>
+      <c r="H11" s="14" t="s">
         <v>91</v>
       </c>
-      <c r="G11" s="14" t="s">
-        <v>75</v>
-      </c>
-      <c r="H11" s="14" t="s">
-        <v>92</v>
-      </c>
       <c r="I11" s="14" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="J11" s="14"/>
       <c r="K11" s="14">
         <v>2021</v>
       </c>
       <c r="L11" s="17" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="M11" s="18"/>
       <c r="N11" s="18"/>
@@ -27829,7 +27829,7 @@
     </row>
     <row r="12" spans="1:26" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A12" s="14" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="B12" s="15">
         <v>12.74245</v>
@@ -27844,25 +27844,25 @@
         <v>11</v>
       </c>
       <c r="F12" s="14" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="G12" s="14" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="H12" s="14" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="I12" s="14">
         <v>1000000</v>
       </c>
       <c r="J12" s="14" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="K12" s="14">
         <v>2021</v>
       </c>
       <c r="L12" s="17" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="M12" s="18"/>
       <c r="N12" s="18"/>
@@ -27881,7 +27881,7 @@
     </row>
     <row r="13" spans="1:26" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A13" s="14" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
       <c r="B13" s="15">
         <v>9.7164300000000008</v>
@@ -27896,13 +27896,13 @@
         <v>11</v>
       </c>
       <c r="F13" s="14" t="s">
+        <v>73</v>
+      </c>
+      <c r="G13" s="14" t="s">
         <v>74</v>
       </c>
-      <c r="G13" s="14" t="s">
-        <v>75</v>
-      </c>
       <c r="H13" s="14" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
       <c r="I13" s="14">
         <v>1000000</v>
@@ -27912,7 +27912,7 @@
         <v>2021</v>
       </c>
       <c r="L13" s="17" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="M13" s="18"/>
       <c r="N13" s="18"/>
@@ -27931,7 +27931,7 @@
     </row>
     <row r="14" spans="1:26" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A14" s="14" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="B14" s="15">
         <v>9.8099799999999995</v>
@@ -27946,25 +27946,25 @@
         <v>11</v>
       </c>
       <c r="F14" s="14" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="G14" s="14" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="H14" s="14" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="I14" s="14">
         <v>1300000</v>
       </c>
       <c r="J14" s="14" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="K14" s="14">
         <v>2021</v>
       </c>
       <c r="L14" s="17" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="M14" s="18"/>
       <c r="N14" s="18"/>
@@ -27999,10 +27999,10 @@
       </c>
       <c r="F15" s="14"/>
       <c r="G15" s="14" t="s">
+        <v>96</v>
+      </c>
+      <c r="H15" s="14" t="s">
         <v>97</v>
-      </c>
-      <c r="H15" s="14" t="s">
-        <v>98</v>
       </c>
       <c r="I15" s="14"/>
       <c r="J15" s="14"/>
@@ -28010,7 +28010,7 @@
         <v>2021</v>
       </c>
       <c r="L15" s="17" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="M15" s="18"/>
       <c r="N15" s="18"/>
@@ -28044,13 +28044,13 @@
         <v>18</v>
       </c>
       <c r="F16" s="14" t="s">
+        <v>98</v>
+      </c>
+      <c r="G16" s="14" t="s">
+        <v>96</v>
+      </c>
+      <c r="H16" s="14" t="s">
         <v>99</v>
-      </c>
-      <c r="G16" s="14" t="s">
-        <v>97</v>
-      </c>
-      <c r="H16" s="14" t="s">
-        <v>100</v>
       </c>
       <c r="I16" s="14"/>
       <c r="J16" s="14"/>
@@ -28058,7 +28058,7 @@
         <v>2021</v>
       </c>
       <c r="L16" s="17" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="M16" s="18"/>
       <c r="N16" s="18"/>
@@ -28092,13 +28092,13 @@
         <v>18</v>
       </c>
       <c r="F17" s="14" t="s">
+        <v>100</v>
+      </c>
+      <c r="G17" s="14" t="s">
+        <v>96</v>
+      </c>
+      <c r="H17" s="14" t="s">
         <v>101</v>
-      </c>
-      <c r="G17" s="14" t="s">
-        <v>97</v>
-      </c>
-      <c r="H17" s="14" t="s">
-        <v>102</v>
       </c>
       <c r="I17" s="14"/>
       <c r="J17" s="14"/>
@@ -28106,7 +28106,7 @@
         <v>2021</v>
       </c>
       <c r="L17" s="17" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="M17" s="18"/>
       <c r="N17" s="18"/>
@@ -28125,7 +28125,7 @@
     </row>
     <row r="18" spans="1:26" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A18" s="14" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="B18" s="15">
         <v>11.924099999999999</v>
@@ -28140,25 +28140,25 @@
         <v>9</v>
       </c>
       <c r="F18" s="14" t="s">
+        <v>102</v>
+      </c>
+      <c r="G18" s="14" t="s">
         <v>103</v>
       </c>
-      <c r="G18" s="14" t="s">
+      <c r="H18" s="14" t="s">
         <v>104</v>
-      </c>
-      <c r="H18" s="14" t="s">
-        <v>105</v>
       </c>
       <c r="I18" s="14">
         <v>600</v>
       </c>
       <c r="J18" s="14" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="K18" s="14">
         <v>2021</v>
       </c>
       <c r="L18" s="17" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="M18" s="18"/>
       <c r="N18" s="18"/>
@@ -28177,7 +28177,7 @@
     </row>
     <row r="19" spans="1:26" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A19" s="14" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="B19" s="15">
         <v>11.053699999999999</v>
@@ -28192,25 +28192,25 @@
         <v>9</v>
       </c>
       <c r="F19" s="14" t="s">
+        <v>106</v>
+      </c>
+      <c r="G19" s="14" t="s">
+        <v>103</v>
+      </c>
+      <c r="H19" s="14" t="s">
         <v>107</v>
-      </c>
-      <c r="G19" s="14" t="s">
-        <v>104</v>
-      </c>
-      <c r="H19" s="14" t="s">
-        <v>108</v>
       </c>
       <c r="I19" s="14">
         <v>180000</v>
       </c>
       <c r="J19" s="14" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="K19" s="14" t="s">
+        <v>108</v>
+      </c>
+      <c r="L19" s="14" t="s">
         <v>109</v>
-      </c>
-      <c r="L19" s="14" t="s">
-        <v>110</v>
       </c>
       <c r="M19" s="18"/>
       <c r="N19" s="18"/>
@@ -28229,7 +28229,7 @@
     </row>
     <row r="20" spans="1:26" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A20" s="14" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="B20" s="15">
         <v>11.30925</v>
@@ -28244,25 +28244,25 @@
         <v>9</v>
       </c>
       <c r="F20" s="14" t="s">
+        <v>110</v>
+      </c>
+      <c r="G20" s="14" t="s">
+        <v>103</v>
+      </c>
+      <c r="H20" s="14" t="s">
         <v>111</v>
-      </c>
-      <c r="G20" s="14" t="s">
-        <v>104</v>
-      </c>
-      <c r="H20" s="14" t="s">
-        <v>112</v>
       </c>
       <c r="I20" s="14">
         <v>130000</v>
       </c>
       <c r="J20" s="14" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="K20" s="14" t="s">
+        <v>108</v>
+      </c>
+      <c r="L20" s="14" t="s">
         <v>109</v>
-      </c>
-      <c r="L20" s="14" t="s">
-        <v>110</v>
       </c>
       <c r="M20" s="18"/>
       <c r="N20" s="18"/>
@@ -28296,25 +28296,25 @@
         <v>9</v>
       </c>
       <c r="F21" s="14" t="s">
+        <v>112</v>
+      </c>
+      <c r="G21" s="14" t="s">
+        <v>103</v>
+      </c>
+      <c r="H21" s="14" t="s">
         <v>113</v>
-      </c>
-      <c r="G21" s="14" t="s">
-        <v>104</v>
-      </c>
-      <c r="H21" s="14" t="s">
-        <v>114</v>
       </c>
       <c r="I21" s="14">
         <v>421000</v>
       </c>
       <c r="J21" s="14" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="K21" s="14">
         <v>2021</v>
       </c>
       <c r="L21" s="17" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="M21" s="18"/>
       <c r="N21" s="18"/>
@@ -28333,7 +28333,7 @@
     </row>
     <row r="22" spans="1:26" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A22" s="14" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="B22" s="15">
         <v>10.20872</v>
@@ -28348,25 +28348,25 @@
         <v>9</v>
       </c>
       <c r="F22" s="14" t="s">
+        <v>114</v>
+      </c>
+      <c r="G22" s="14" t="s">
+        <v>103</v>
+      </c>
+      <c r="H22" s="14" t="s">
         <v>115</v>
-      </c>
-      <c r="G22" s="14" t="s">
-        <v>104</v>
-      </c>
-      <c r="H22" s="14" t="s">
-        <v>116</v>
       </c>
       <c r="I22" s="14">
         <v>730000</v>
       </c>
       <c r="J22" s="14" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="K22" s="14">
         <v>2022</v>
       </c>
       <c r="L22" s="14" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
       <c r="M22" s="18"/>
       <c r="N22" s="18"/>
@@ -28400,25 +28400,25 @@
         <v>9</v>
       </c>
       <c r="F23" s="14" t="s">
+        <v>117</v>
+      </c>
+      <c r="G23" s="14" t="s">
+        <v>103</v>
+      </c>
+      <c r="H23" s="14" t="s">
         <v>118</v>
-      </c>
-      <c r="G23" s="14" t="s">
-        <v>104</v>
-      </c>
-      <c r="H23" s="14" t="s">
-        <v>119</v>
       </c>
       <c r="I23" s="14">
         <v>110000</v>
       </c>
       <c r="J23" s="14" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="K23" s="14" t="s">
+        <v>108</v>
+      </c>
+      <c r="L23" s="14" t="s">
         <v>109</v>
-      </c>
-      <c r="L23" s="14" t="s">
-        <v>110</v>
       </c>
       <c r="M23" s="18"/>
       <c r="N23" s="18"/>
@@ -28452,25 +28452,25 @@
         <v>9</v>
       </c>
       <c r="F24" s="14" t="s">
+        <v>119</v>
+      </c>
+      <c r="G24" s="14" t="s">
+        <v>103</v>
+      </c>
+      <c r="H24" s="14" t="s">
         <v>120</v>
-      </c>
-      <c r="G24" s="14" t="s">
-        <v>104</v>
-      </c>
-      <c r="H24" s="14" t="s">
-        <v>121</v>
       </c>
       <c r="I24" s="14">
         <v>93000</v>
       </c>
       <c r="J24" s="14" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="K24" s="14">
         <v>2021</v>
       </c>
       <c r="L24" s="17" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="M24" s="18"/>
       <c r="N24" s="18"/>
@@ -28504,25 +28504,25 @@
         <v>9</v>
       </c>
       <c r="F25" s="14" t="s">
+        <v>121</v>
+      </c>
+      <c r="G25" s="14" t="s">
+        <v>103</v>
+      </c>
+      <c r="H25" s="14" t="s">
         <v>122</v>
-      </c>
-      <c r="G25" s="14" t="s">
-        <v>104</v>
-      </c>
-      <c r="H25" s="14" t="s">
-        <v>123</v>
       </c>
       <c r="I25" s="14">
         <v>150000</v>
       </c>
       <c r="J25" s="14" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="K25" s="14">
         <v>2021</v>
       </c>
       <c r="L25" s="17" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="M25" s="18"/>
       <c r="N25" s="18"/>
@@ -28556,25 +28556,25 @@
         <v>9</v>
       </c>
       <c r="F26" s="14" t="s">
+        <v>123</v>
+      </c>
+      <c r="G26" s="14" t="s">
+        <v>103</v>
+      </c>
+      <c r="H26" s="14" t="s">
         <v>124</v>
-      </c>
-      <c r="G26" s="14" t="s">
-        <v>104</v>
-      </c>
-      <c r="H26" s="14" t="s">
-        <v>125</v>
       </c>
       <c r="I26" s="14">
         <v>100000</v>
       </c>
       <c r="J26" s="14" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="K26" s="14" t="s">
+        <v>108</v>
+      </c>
+      <c r="L26" s="14" t="s">
         <v>109</v>
-      </c>
-      <c r="L26" s="14" t="s">
-        <v>110</v>
       </c>
       <c r="M26" s="18"/>
       <c r="N26" s="18"/>
@@ -28608,25 +28608,25 @@
         <v>9</v>
       </c>
       <c r="F27" s="14" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
       <c r="G27" s="14" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="H27" s="14" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="I27" s="14">
         <v>540000</v>
       </c>
       <c r="J27" s="14" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="K27" s="14">
         <v>2021</v>
       </c>
       <c r="L27" s="17" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="M27" s="18"/>
       <c r="N27" s="18"/>
@@ -28660,25 +28660,25 @@
         <v>9</v>
       </c>
       <c r="F28" s="14" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
       <c r="G28" s="14" t="s">
+        <v>126</v>
+      </c>
+      <c r="H28" s="14" t="s">
         <v>127</v>
-      </c>
-      <c r="H28" s="14" t="s">
-        <v>128</v>
       </c>
       <c r="I28" s="14">
         <v>160000</v>
       </c>
       <c r="J28" s="14" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="K28" s="14" t="s">
+        <v>108</v>
+      </c>
+      <c r="L28" s="14" t="s">
         <v>109</v>
-      </c>
-      <c r="L28" s="14" t="s">
-        <v>110</v>
       </c>
       <c r="M28" s="18"/>
       <c r="N28" s="18"/>
@@ -28712,25 +28712,25 @@
         <v>9</v>
       </c>
       <c r="F29" s="14" t="s">
+        <v>128</v>
+      </c>
+      <c r="G29" s="14" t="s">
+        <v>103</v>
+      </c>
+      <c r="H29" s="14" t="s">
         <v>129</v>
-      </c>
-      <c r="G29" s="14" t="s">
-        <v>104</v>
-      </c>
-      <c r="H29" s="14" t="s">
-        <v>130</v>
       </c>
       <c r="I29" s="14">
         <v>174900</v>
       </c>
       <c r="J29" s="14" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="K29" s="14">
         <v>2021</v>
       </c>
       <c r="L29" s="17" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="M29" s="18"/>
       <c r="N29" s="18"/>
@@ -28764,25 +28764,25 @@
         <v>9</v>
       </c>
       <c r="F30" s="14" t="s">
+        <v>130</v>
+      </c>
+      <c r="G30" s="14" t="s">
+        <v>103</v>
+      </c>
+      <c r="H30" s="14" t="s">
         <v>131</v>
-      </c>
-      <c r="G30" s="14" t="s">
-        <v>104</v>
-      </c>
-      <c r="H30" s="14" t="s">
-        <v>132</v>
       </c>
       <c r="I30" s="14">
         <v>93400</v>
       </c>
       <c r="J30" s="14" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="K30" s="14">
         <v>2021</v>
       </c>
       <c r="L30" s="17" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="M30" s="18"/>
       <c r="N30" s="18"/>
@@ -28801,7 +28801,7 @@
     </row>
     <row r="31" spans="1:26" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A31" s="14" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="B31" s="15">
         <v>13.80006</v>
@@ -28816,25 +28816,25 @@
         <v>9</v>
       </c>
       <c r="F31" s="14" t="s">
+        <v>102</v>
+      </c>
+      <c r="G31" s="14" t="s">
         <v>103</v>
       </c>
-      <c r="G31" s="14" t="s">
-        <v>104</v>
-      </c>
       <c r="H31" s="14" t="s">
-        <v>133</v>
+        <v>132</v>
       </c>
       <c r="I31" s="14">
         <v>612</v>
       </c>
       <c r="J31" s="14" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="K31" s="14">
         <v>2021</v>
       </c>
       <c r="L31" s="17" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="M31" s="18"/>
       <c r="N31" s="18"/>
@@ -28853,7 +28853,7 @@
     </row>
     <row r="32" spans="1:26" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A32" s="14" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="B32" s="15">
         <v>12.63189</v>
@@ -28868,25 +28868,25 @@
         <v>9</v>
       </c>
       <c r="F32" s="14" t="s">
+        <v>133</v>
+      </c>
+      <c r="G32" s="14" t="s">
+        <v>103</v>
+      </c>
+      <c r="H32" s="14" t="s">
         <v>134</v>
-      </c>
-      <c r="G32" s="14" t="s">
-        <v>104</v>
-      </c>
-      <c r="H32" s="14" t="s">
-        <v>135</v>
       </c>
       <c r="I32" s="14">
         <v>150000</v>
       </c>
       <c r="J32" s="14" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="K32" s="14">
         <v>2021</v>
       </c>
       <c r="L32" s="17" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="M32" s="18"/>
       <c r="N32" s="18"/>
@@ -28905,7 +28905,7 @@
     </row>
     <row r="33" spans="1:26" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A33" s="14" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="B33" s="15">
         <v>11.556369999999999</v>
@@ -28920,25 +28920,25 @@
         <v>9</v>
       </c>
       <c r="F33" s="14" t="s">
-        <v>134</v>
+        <v>133</v>
       </c>
       <c r="G33" s="14" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="H33" s="14" t="s">
-        <v>136</v>
+        <v>135</v>
       </c>
       <c r="I33" s="14">
         <v>153333.33333333331</v>
       </c>
       <c r="J33" s="14" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="K33" s="14">
         <v>2021</v>
       </c>
       <c r="L33" s="17" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="M33" s="18"/>
       <c r="N33" s="18"/>
@@ -28957,7 +28957,7 @@
     </row>
     <row r="34" spans="1:26" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A34" s="14" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="B34" s="15">
         <v>12.08798</v>
@@ -28972,25 +28972,25 @@
         <v>9</v>
       </c>
       <c r="F34" s="14" t="s">
-        <v>134</v>
+        <v>133</v>
       </c>
       <c r="G34" s="14" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="H34" s="14" t="s">
-        <v>137</v>
+        <v>136</v>
       </c>
       <c r="I34" s="14">
         <v>120000</v>
       </c>
       <c r="J34" s="14" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="K34" s="14">
         <v>2021</v>
       </c>
       <c r="L34" s="17" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="M34" s="18"/>
       <c r="N34" s="18"/>
@@ -29009,7 +29009,7 @@
     </row>
     <row r="35" spans="1:26" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A35" s="14" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="B35" s="15">
         <v>11.428890000000001</v>
@@ -29024,25 +29024,25 @@
         <v>9</v>
       </c>
       <c r="F35" s="14" t="s">
+        <v>137</v>
+      </c>
+      <c r="G35" s="14" t="s">
+        <v>103</v>
+      </c>
+      <c r="H35" s="14" t="s">
         <v>138</v>
-      </c>
-      <c r="G35" s="14" t="s">
-        <v>104</v>
-      </c>
-      <c r="H35" s="14" t="s">
-        <v>139</v>
       </c>
       <c r="I35" s="14">
         <v>222000</v>
       </c>
       <c r="J35" s="14" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="K35" s="14">
         <v>2021</v>
       </c>
       <c r="L35" s="17" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="M35" s="18"/>
       <c r="N35" s="18"/>
@@ -29061,7 +29061,7 @@
     </row>
     <row r="36" spans="1:26" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A36" s="14" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="B36" s="15">
         <v>10.943759999999999</v>
@@ -29076,25 +29076,25 @@
         <v>9</v>
       </c>
       <c r="F36" s="14" t="s">
-        <v>134</v>
+        <v>133</v>
       </c>
       <c r="G36" s="14" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="H36" s="14" t="s">
-        <v>140</v>
+        <v>139</v>
       </c>
       <c r="I36" s="14">
         <v>203125</v>
       </c>
       <c r="J36" s="14" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="K36" s="14">
         <v>2021</v>
       </c>
       <c r="L36" s="17" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="M36" s="18"/>
       <c r="N36" s="18"/>
@@ -29113,7 +29113,7 @@
     </row>
     <row r="37" spans="1:26" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A37" s="14" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="B37" s="15">
         <v>10.35805</v>
@@ -29128,25 +29128,25 @@
         <v>9</v>
       </c>
       <c r="F37" s="14" t="s">
+        <v>140</v>
+      </c>
+      <c r="G37" s="14" t="s">
         <v>141</v>
       </c>
-      <c r="G37" s="14" t="s">
+      <c r="H37" s="14" t="s">
         <v>142</v>
-      </c>
-      <c r="H37" s="14" t="s">
-        <v>143</v>
       </c>
       <c r="I37" s="14">
         <v>195000</v>
       </c>
       <c r="J37" s="14" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="K37" s="14">
         <v>2021</v>
       </c>
       <c r="L37" s="17" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="M37" s="18"/>
       <c r="N37" s="18"/>
@@ -29180,25 +29180,25 @@
         <v>9</v>
       </c>
       <c r="F38" s="14" t="s">
+        <v>143</v>
+      </c>
+      <c r="G38" s="14" t="s">
+        <v>103</v>
+      </c>
+      <c r="H38" s="14" t="s">
         <v>144</v>
-      </c>
-      <c r="G38" s="14" t="s">
-        <v>104</v>
-      </c>
-      <c r="H38" s="14" t="s">
-        <v>145</v>
       </c>
       <c r="I38" s="14">
         <v>380000</v>
       </c>
       <c r="J38" s="14" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="K38" s="14">
         <v>2021</v>
       </c>
       <c r="L38" s="17" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="M38" s="18"/>
       <c r="N38" s="18"/>
@@ -29217,7 +29217,7 @@
     </row>
     <row r="39" spans="1:26" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A39" s="14" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
       <c r="B39" s="15">
         <v>9.7325099999999996</v>
@@ -29232,25 +29232,25 @@
         <v>9</v>
       </c>
       <c r="F39" s="14" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="G39" s="14" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="H39" s="14" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
       <c r="I39" s="14">
         <v>120000</v>
       </c>
       <c r="J39" s="14" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="K39" s="14">
         <v>2021</v>
       </c>
       <c r="L39" s="17" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="M39" s="18"/>
       <c r="N39" s="18"/>
@@ -29271,18 +29271,18 @@
     <row r="41" spans="1:26" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
     <row r="42" spans="1:26" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A42" s="12" t="s">
-        <v>147</v>
+        <v>146</v>
       </c>
       <c r="B42" s="19" t="s">
+        <v>57</v>
+      </c>
+      <c r="C42" s="19" t="s">
         <v>58</v>
-      </c>
-      <c r="C42" s="19" t="s">
-        <v>59</v>
       </c>
     </row>
     <row r="43" spans="1:26" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A43" s="1" t="s">
-        <v>148</v>
+        <v>147</v>
       </c>
       <c r="B43" s="4">
         <v>12.053710000000001</v>
@@ -29293,7 +29293,7 @@
     </row>
     <row r="44" spans="1:26" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A44" s="1" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="B44" s="4">
         <v>11.69642</v>
@@ -29304,7 +29304,7 @@
     </row>
     <row r="45" spans="1:26" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A45" s="1" t="s">
-        <v>149</v>
+        <v>148</v>
       </c>
       <c r="B45" s="4">
         <v>10.748810000000001</v>
@@ -29315,7 +29315,7 @@
     </row>
     <row r="46" spans="1:26" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A46" s="1" t="s">
-        <v>150</v>
+        <v>149</v>
       </c>
       <c r="B46" s="4">
         <v>9.0727600000000006</v>
@@ -29337,7 +29337,7 @@
     </row>
     <row r="48" spans="1:26" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A48" s="1" t="s">
-        <v>151</v>
+        <v>150</v>
       </c>
       <c r="B48" s="4">
         <v>8.3271999999999995</v>
@@ -29348,7 +29348,7 @@
     </row>
     <row r="49" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A49" s="1" t="s">
-        <v>152</v>
+        <v>151</v>
       </c>
       <c r="B49" s="4">
         <v>8.6266800000000003</v>
@@ -29359,7 +29359,7 @@
     </row>
     <row r="50" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A50" s="1" t="s">
-        <v>153</v>
+        <v>152</v>
       </c>
       <c r="B50" s="4">
         <v>8.4164499999999993</v>
@@ -29370,7 +29370,7 @@
     </row>
     <row r="51" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A51" s="1" t="s">
-        <v>154</v>
+        <v>153</v>
       </c>
       <c r="B51" s="4">
         <v>9.1895100000000003</v>
@@ -29381,7 +29381,7 @@
     </row>
     <row r="52" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A52" s="1" t="s">
-        <v>155</v>
+        <v>154</v>
       </c>
       <c r="B52" s="4">
         <v>7.6868600000000002</v>
@@ -29392,7 +29392,7 @@
     </row>
     <row r="53" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A53" s="1" t="s">
-        <v>156</v>
+        <v>155</v>
       </c>
       <c r="B53" s="4">
         <v>8.9330499999999997</v>
@@ -29403,7 +29403,7 @@
     </row>
     <row r="54" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A54" s="1" t="s">
-        <v>157</v>
+        <v>156</v>
       </c>
       <c r="B54" s="4">
         <v>10.991619999999999</v>
@@ -29414,7 +29414,7 @@
     </row>
     <row r="55" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A55" s="1" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
       <c r="B55" s="4">
         <v>11.338749999999999</v>
@@ -29425,7 +29425,7 @@
     </row>
     <row r="56" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A56" s="1" t="s">
-        <v>159</v>
+        <v>158</v>
       </c>
       <c r="B56" s="4">
         <v>13.77692</v>
@@ -29436,7 +29436,7 @@
     </row>
     <row r="57" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A57" s="1" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="B57" s="4">
         <v>12.31551</v>
@@ -29459,18 +29459,18 @@
     <row r="59" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
     <row r="60" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A60" s="22" t="s">
-        <v>160</v>
+        <v>159</v>
       </c>
       <c r="B60" s="23" t="s">
+        <v>57</v>
+      </c>
+      <c r="C60" s="23" t="s">
         <v>58</v>
-      </c>
-      <c r="C60" s="23" t="s">
-        <v>59</v>
       </c>
     </row>
     <row r="61" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A61" s="21" t="s">
-        <v>161</v>
+        <v>160</v>
       </c>
       <c r="B61" s="2">
         <v>12.274480000000001</v>
@@ -29482,18 +29482,18 @@
     <row r="62" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
     <row r="63" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A63" s="23" t="s">
-        <v>162</v>
+        <v>161</v>
       </c>
       <c r="B63" s="23" t="s">
+        <v>57</v>
+      </c>
+      <c r="C63" s="23" t="s">
         <v>58</v>
-      </c>
-      <c r="C63" s="23" t="s">
-        <v>59</v>
       </c>
     </row>
     <row r="64" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A64" s="4" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="B64" s="4">
         <v>10.64</v>

</xml_diff>

<commit_message>
changed node_metrics fluxes from kg to t
</commit_message>
<xml_diff>
--- a/southern_europe/italy_data/geographical_feature/node_metrics.xlsx
+++ b/southern_europe/italy_data/geographical_feature/node_metrics.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\0954659\PycharmProjects\AdOpT-NET0_luca\southern_europe\italy_data\geographical_feature\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2B3C1B2B-48C0-4613-8342-018C8D2C2E2B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E6818FCA-ECDD-428E-8F98-1F6452D13D4F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="22932" yWindow="-4368" windowWidth="30936" windowHeight="16776" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="nodes" sheetId="1" r:id="rId1"/>
@@ -20,10 +20,6 @@
     <sheet name="raw_data" sheetId="5" r:id="rId5"/>
     <sheet name="readme" sheetId="6" r:id="rId6"/>
   </sheets>
-  <externalReferences>
-    <externalReference r:id="rId7"/>
-    <externalReference r:id="rId8"/>
-  </externalReferences>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">nodes!$H$1:$H$46</definedName>
   </definedNames>
@@ -700,36 +696,6 @@
 </styleSheet>
 </file>
 
-<file path=xl/externalLinks/externalLink1.xml><?xml version="1.0" encoding="utf-8"?>
-<externalLink xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xxl21="http://schemas.microsoft.com/office/spreadsheetml/2021/extlinks2021" mc:Ignorable="x14 xxl21">
-  <externalBook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1">
-    <sheetNames>
-      <sheetName val="Waste - TERMOVALORIZZATORE COMO"/>
-    </sheetNames>
-    <sheetDataSet>
-      <sheetData sheetId="0" refreshError="1"/>
-    </sheetDataSet>
-  </externalBook>
-</externalLink>
-</file>
-
-<file path=xl/externalLinks/externalLink2.xml><?xml version="1.0" encoding="utf-8"?>
-<externalLink xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xxl21="http://schemas.microsoft.com/office/spreadsheetml/2021/extlinks2021" mc:Ignorable="x14 xxl21">
-  <externalBook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1">
-    <sheetNames>
-      <sheetName val="Waste - SILLA 2"/>
-      <sheetName val="Waste -  PIACENZA Iren"/>
-      <sheetName val="Cement-VERNASCA"/>
-    </sheetNames>
-    <sheetDataSet>
-      <sheetData sheetId="0" refreshError="1"/>
-      <sheetData sheetId="1" refreshError="1"/>
-      <sheetData sheetId="2" refreshError="1"/>
-    </sheetDataSet>
-  </externalBook>
-</externalLink>
-</file>
-
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
 <a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Sheets">
   <a:themeElements>
@@ -982,8 +948,11 @@
       <c r="E2" s="4">
         <v>10</v>
       </c>
-      <c r="F2" s="3">
-        <v>600525753</v>
+      <c r="F2">
+        <v>600525.75300000003</v>
+      </c>
+      <c r="G2">
+        <v>0</v>
       </c>
       <c r="H2" s="1" t="s">
         <v>9</v>
@@ -1005,8 +974,11 @@
       <c r="E3" s="4">
         <v>10</v>
       </c>
-      <c r="F3" s="3">
-        <v>933726000</v>
+      <c r="F3">
+        <v>933726</v>
+      </c>
+      <c r="G3">
+        <v>0</v>
       </c>
       <c r="H3" s="1" t="s">
         <v>11</v>
@@ -1028,7 +1000,10 @@
       <c r="E4" s="4">
         <v>10</v>
       </c>
-      <c r="F4" s="4">
+      <c r="F4">
+        <v>0</v>
+      </c>
+      <c r="G4">
         <v>0</v>
       </c>
       <c r="H4" s="1" t="s">
@@ -1051,8 +1026,11 @@
       <c r="E5" s="4">
         <v>10</v>
       </c>
-      <c r="F5" s="3">
-        <v>510739000</v>
+      <c r="F5">
+        <v>510739</v>
+      </c>
+      <c r="G5">
+        <v>0</v>
       </c>
       <c r="H5" s="1" t="s">
         <v>11</v>
@@ -1074,8 +1052,11 @@
       <c r="E6" s="4">
         <v>10</v>
       </c>
-      <c r="F6" s="3">
-        <v>536971000</v>
+      <c r="F6">
+        <v>536971</v>
+      </c>
+      <c r="G6">
+        <v>0</v>
       </c>
       <c r="H6" s="1" t="s">
         <v>11</v>
@@ -1097,8 +1078,11 @@
       <c r="E7" s="4">
         <v>10</v>
       </c>
-      <c r="F7" s="3">
-        <v>122771831.36135496</v>
+      <c r="F7">
+        <v>122771.83136135497</v>
+      </c>
+      <c r="G7">
+        <v>0</v>
       </c>
       <c r="H7" s="1" t="s">
         <v>9</v>
@@ -1120,8 +1104,11 @@
       <c r="E8" s="4">
         <v>10</v>
       </c>
-      <c r="F8" s="3">
-        <v>850236000</v>
+      <c r="F8">
+        <v>850236</v>
+      </c>
+      <c r="G8">
+        <v>0</v>
       </c>
       <c r="H8" s="1" t="s">
         <v>18</v>
@@ -1143,8 +1130,11 @@
       <c r="E9" s="4">
         <v>10</v>
       </c>
-      <c r="F9" s="3">
-        <v>338516000</v>
+      <c r="F9">
+        <v>338516</v>
+      </c>
+      <c r="G9">
+        <v>0</v>
       </c>
       <c r="H9" s="1" t="s">
         <v>9</v>
@@ -1166,10 +1156,12 @@
       <c r="E10" s="4">
         <v>10</v>
       </c>
-      <c r="F10" s="3">
-        <v>1597264000</v>
-      </c>
-      <c r="G10" s="1"/>
+      <c r="F10">
+        <v>1597264</v>
+      </c>
+      <c r="G10">
+        <v>0</v>
+      </c>
       <c r="H10" s="1" t="s">
         <v>18</v>
       </c>
@@ -1190,8 +1182,11 @@
       <c r="E11" s="4">
         <v>10</v>
       </c>
-      <c r="F11" s="3">
-        <v>258516117</v>
+      <c r="F11">
+        <v>258516.117</v>
+      </c>
+      <c r="G11">
+        <v>0</v>
       </c>
       <c r="H11" s="1" t="s">
         <v>18</v>
@@ -1213,11 +1208,10 @@
       <c r="E12" s="4">
         <v>10</v>
       </c>
-      <c r="F12" s="3">
-        <v>105538400</v>
-      </c>
-      <c r="G12" s="3">
-        <f>SUM('[1]Waste - TERMOVALORIZZATORE COMO'!$C$3:$C$17522)*1000</f>
+      <c r="F12">
+        <v>105538.4</v>
+      </c>
+      <c r="G12">
         <v>0</v>
       </c>
       <c r="H12" s="1" t="s">
@@ -1240,8 +1234,11 @@
       <c r="E13" s="4">
         <v>10</v>
       </c>
-      <c r="F13" s="3">
-        <v>111610755.78304997</v>
+      <c r="F13">
+        <v>111610.75578304997</v>
+      </c>
+      <c r="G13">
+        <v>0</v>
       </c>
       <c r="H13" s="1" t="s">
         <v>9</v>
@@ -1263,11 +1260,10 @@
       <c r="E14" s="4">
         <v>10</v>
       </c>
-      <c r="F14" s="3">
-        <v>323606842</v>
-      </c>
-      <c r="G14" s="3">
-        <f>SUM('[2]Waste - SILLA 2'!$C$3:$C$8761)*1000</f>
+      <c r="F14">
+        <v>323606.842</v>
+      </c>
+      <c r="G14">
         <v>0</v>
       </c>
       <c r="H14" s="1" t="s">
@@ -1290,8 +1286,11 @@
       <c r="E15" s="4">
         <v>10</v>
       </c>
-      <c r="F15" s="3">
-        <v>223853000</v>
+      <c r="F15">
+        <v>223853</v>
+      </c>
+      <c r="G15">
+        <v>0</v>
       </c>
       <c r="H15" s="1" t="s">
         <v>9</v>
@@ -1313,7 +1312,10 @@
       <c r="E16" s="4">
         <v>10</v>
       </c>
-      <c r="F16" s="3">
+      <c r="F16">
+        <v>0</v>
+      </c>
+      <c r="G16">
         <v>0</v>
       </c>
       <c r="H16" s="1" t="s">
@@ -1336,8 +1338,11 @@
       <c r="E17" s="4">
         <v>10</v>
       </c>
-      <c r="F17" s="3">
-        <v>120000000</v>
+      <c r="F17">
+        <v>120000</v>
+      </c>
+      <c r="G17">
+        <v>0</v>
       </c>
       <c r="H17" s="1" t="s">
         <v>9</v>
@@ -1359,8 +1364,11 @@
       <c r="E18" s="4">
         <v>10</v>
       </c>
-      <c r="F18" s="3">
-        <v>128208990</v>
+      <c r="F18">
+        <v>128208.99</v>
+      </c>
+      <c r="G18">
+        <v>0</v>
       </c>
       <c r="H18" s="1" t="s">
         <v>9</v>
@@ -1382,8 +1390,11 @@
       <c r="E19" s="4">
         <v>10</v>
       </c>
-      <c r="F19" s="3">
-        <v>790120000</v>
+      <c r="F19">
+        <v>790120</v>
+      </c>
+      <c r="G19">
+        <v>0</v>
       </c>
       <c r="H19" s="1" t="s">
         <v>11</v>
@@ -1405,8 +1416,11 @@
       <c r="E20" s="4">
         <v>10</v>
       </c>
-      <c r="F20" s="3">
-        <v>190599884</v>
+      <c r="F20">
+        <v>190599.88399999999</v>
+      </c>
+      <c r="G20">
+        <v>0</v>
       </c>
       <c r="H20" s="1" t="s">
         <v>9</v>
@@ -1428,11 +1442,10 @@
       <c r="E21" s="6">
         <v>10</v>
       </c>
-      <c r="F21" s="3">
-        <v>123636000</v>
-      </c>
-      <c r="G21" s="3">
-        <f>SUM('[2]Waste -  PIACENZA Iren'!$C$3:$C$8762)*1000</f>
+      <c r="F21">
+        <v>123636</v>
+      </c>
+      <c r="G21">
         <v>0</v>
       </c>
       <c r="H21" s="1" t="s">
@@ -1455,10 +1468,12 @@
       <c r="E22" s="6">
         <v>10</v>
       </c>
-      <c r="F22" s="3">
-        <v>405887000</v>
-      </c>
-      <c r="G22" s="3"/>
+      <c r="F22">
+        <v>405887</v>
+      </c>
+      <c r="G22">
+        <v>0</v>
+      </c>
       <c r="H22" s="1" t="s">
         <v>11</v>
       </c>
@@ -1479,11 +1494,10 @@
       <c r="E23" s="4">
         <v>10</v>
       </c>
-      <c r="F23" s="3">
-        <v>587138470</v>
-      </c>
-      <c r="G23" s="3">
-        <f>SUM('[2]Cement-VERNASCA'!$C$3:$C$367)*1000</f>
+      <c r="F23">
+        <v>587138.47</v>
+      </c>
+      <c r="G23">
         <v>0</v>
       </c>
       <c r="H23" s="1" t="s">
@@ -1506,8 +1520,11 @@
       <c r="E24" s="4">
         <v>10</v>
       </c>
-      <c r="F24" s="3">
-        <v>128207000</v>
+      <c r="F24">
+        <v>128207</v>
+      </c>
+      <c r="G24">
+        <v>0</v>
       </c>
       <c r="H24" s="1" t="s">
         <v>11</v>
@@ -1529,8 +1546,11 @@
       <c r="E25" s="4">
         <v>10</v>
       </c>
-      <c r="F25" s="3">
-        <v>867256250</v>
+      <c r="F25">
+        <v>867256.25</v>
+      </c>
+      <c r="G25">
+        <v>0</v>
       </c>
       <c r="H25" s="1" t="s">
         <v>9</v>
@@ -1552,8 +1572,11 @@
       <c r="E26" s="4">
         <v>10</v>
       </c>
-      <c r="F26" s="3">
-        <v>918742000</v>
+      <c r="F26">
+        <v>918742</v>
+      </c>
+      <c r="G26">
+        <v>0</v>
       </c>
       <c r="H26" s="1" t="s">
         <v>11</v>
@@ -1575,11 +1598,11 @@
       <c r="E27" s="4">
         <v>10</v>
       </c>
-      <c r="F27" s="3">
-        <v>166966760</v>
-      </c>
-      <c r="G27" s="4">
-        <v>213023660</v>
+      <c r="F27">
+        <v>166966.76</v>
+      </c>
+      <c r="G27">
+        <v>213023.66</v>
       </c>
       <c r="H27" s="1" t="s">
         <v>9</v>
@@ -1601,8 +1624,11 @@
       <c r="E28" s="4">
         <v>10</v>
       </c>
-      <c r="F28" s="3">
-        <v>200899360.40948996</v>
+      <c r="F28">
+        <v>200899.36040948995</v>
+      </c>
+      <c r="G28">
+        <v>0</v>
       </c>
       <c r="H28" s="1" t="s">
         <v>9</v>
@@ -1624,8 +1650,11 @@
       <c r="E29" s="4">
         <v>10</v>
       </c>
-      <c r="F29" s="3">
-        <v>186706873</v>
+      <c r="F29">
+        <v>186706.87299999999</v>
+      </c>
+      <c r="G29">
+        <v>0</v>
       </c>
       <c r="H29" s="1" t="s">
         <v>9</v>
@@ -1647,8 +1676,11 @@
       <c r="E30" s="4">
         <v>10</v>
       </c>
-      <c r="F30" s="3">
-        <v>145093982.51796496</v>
+      <c r="F30">
+        <v>145093.98251796496</v>
+      </c>
+      <c r="G30">
+        <v>0</v>
       </c>
       <c r="H30" s="1" t="s">
         <v>9</v>
@@ -1670,8 +1702,11 @@
       <c r="E31" s="4">
         <v>10</v>
       </c>
-      <c r="F31" s="3">
-        <v>130183000</v>
+      <c r="F31">
+        <v>130183</v>
+      </c>
+      <c r="G31">
+        <v>0</v>
       </c>
       <c r="H31" s="1" t="s">
         <v>9</v>
@@ -1693,8 +1728,11 @@
       <c r="E32" s="4">
         <v>10</v>
       </c>
-      <c r="F32" s="3">
-        <v>186972000</v>
+      <c r="F32">
+        <v>186972</v>
+      </c>
+      <c r="G32">
+        <v>0</v>
       </c>
       <c r="H32" s="1" t="s">
         <v>9</v>
@@ -1716,11 +1754,11 @@
       <c r="E33" s="4">
         <v>10</v>
       </c>
-      <c r="F33" s="3">
-        <v>342306000</v>
-      </c>
-      <c r="G33" s="4">
-        <v>342306000</v>
+      <c r="F33">
+        <v>342306</v>
+      </c>
+      <c r="G33">
+        <v>342306</v>
       </c>
       <c r="H33" s="1" t="s">
         <v>11</v>
@@ -1742,7 +1780,10 @@
       <c r="E34" s="4">
         <v>10</v>
       </c>
-      <c r="F34" s="3">
+      <c r="F34">
+        <v>0</v>
+      </c>
+      <c r="G34">
         <v>0</v>
       </c>
       <c r="H34" s="1" t="s">
@@ -1765,8 +1806,11 @@
       <c r="E35" s="4">
         <v>10</v>
       </c>
-      <c r="F35" s="3">
-        <v>351766000</v>
+      <c r="F35">
+        <v>351766</v>
+      </c>
+      <c r="G35">
+        <v>0</v>
       </c>
       <c r="H35" s="1" t="s">
         <v>11</v>
@@ -1788,8 +1832,11 @@
       <c r="E36" s="4">
         <v>10</v>
       </c>
-      <c r="F36" s="3">
-        <v>179315793</v>
+      <c r="F36">
+        <v>179315.79300000001</v>
+      </c>
+      <c r="G36">
+        <v>0</v>
       </c>
       <c r="H36" s="1" t="s">
         <v>9</v>
@@ -1811,8 +1858,11 @@
       <c r="E37" s="4">
         <v>10</v>
       </c>
-      <c r="F37" s="3">
-        <v>144055000</v>
+      <c r="F37">
+        <v>144055</v>
+      </c>
+      <c r="G37">
+        <v>0</v>
       </c>
       <c r="H37" s="1" t="s">
         <v>9</v>
@@ -1834,8 +1884,11 @@
       <c r="E38" s="4">
         <v>10</v>
       </c>
-      <c r="F38" s="3">
-        <v>197108000</v>
+      <c r="F38">
+        <v>197108</v>
+      </c>
+      <c r="G38">
+        <v>0</v>
       </c>
       <c r="H38" s="1" t="s">
         <v>11</v>
@@ -1857,10 +1910,12 @@
       <c r="E39" s="6">
         <v>10</v>
       </c>
-      <c r="F39" s="3">
-        <v>500000000</v>
-      </c>
-      <c r="G39" s="3"/>
+      <c r="F39">
+        <v>500000</v>
+      </c>
+      <c r="G39">
+        <v>0</v>
+      </c>
       <c r="H39" s="1" t="s">
         <v>48</v>
       </c>
@@ -1881,7 +1936,10 @@
       <c r="E40" s="4">
         <v>10</v>
       </c>
-      <c r="F40" s="3">
+      <c r="F40">
+        <v>0</v>
+      </c>
+      <c r="G40">
         <v>0</v>
       </c>
       <c r="H40" s="1" t="s">
@@ -1904,11 +1962,11 @@
       <c r="E41" s="4">
         <v>10</v>
       </c>
-      <c r="F41" s="3">
-        <v>438034000</v>
-      </c>
-      <c r="G41" s="4">
-        <v>438034000</v>
+      <c r="F41">
+        <v>438034</v>
+      </c>
+      <c r="G41">
+        <v>438034</v>
       </c>
       <c r="H41" s="1" t="s">
         <v>11</v>
@@ -1930,8 +1988,11 @@
       <c r="E42" s="4">
         <v>10</v>
       </c>
-      <c r="F42" s="3">
-        <v>128100192</v>
+      <c r="F42">
+        <v>128100.192</v>
+      </c>
+      <c r="G42">
+        <v>0</v>
       </c>
       <c r="H42" s="1" t="s">
         <v>9</v>
@@ -1953,8 +2014,11 @@
       <c r="E43" s="4">
         <v>10</v>
       </c>
-      <c r="F43" s="3">
-        <v>157981171</v>
+      <c r="F43">
+        <v>157981.171</v>
+      </c>
+      <c r="G43">
+        <v>0</v>
       </c>
       <c r="H43" s="1" t="s">
         <v>9</v>
@@ -1976,10 +2040,12 @@
       <c r="E44" s="6">
         <v>10</v>
       </c>
-      <c r="F44" s="3">
-        <v>0</v>
-      </c>
-      <c r="G44" s="3"/>
+      <c r="F44">
+        <v>0</v>
+      </c>
+      <c r="G44">
+        <v>0</v>
+      </c>
       <c r="H44" s="1" t="s">
         <v>13</v>
       </c>
@@ -2000,10 +2066,12 @@
       <c r="E45" s="6">
         <v>10</v>
       </c>
-      <c r="F45" s="7">
-        <v>0</v>
-      </c>
-      <c r="G45" s="7"/>
+      <c r="F45">
+        <v>0</v>
+      </c>
+      <c r="G45">
+        <v>0</v>
+      </c>
       <c r="H45" s="1" t="s">
         <v>54</v>
       </c>
@@ -2024,10 +2092,12 @@
       <c r="E46" s="4">
         <v>10</v>
       </c>
-      <c r="F46" s="4">
-        <v>0</v>
-      </c>
-      <c r="G46" s="4"/>
+      <c r="F46">
+        <v>0</v>
+      </c>
+      <c r="G46">
+        <v>0</v>
+      </c>
       <c r="H46" s="4" t="s">
         <v>13</v>
       </c>
@@ -19145,958 +19215,958 @@
     <row r="46" spans="1:45" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
     <row r="47" spans="1:45" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
     <row r="48" spans="1:45" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="49" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="50" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="51" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="52" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="53" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="54" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="55" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="56" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="57" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="58" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="59" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="60" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="61" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="62" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="63" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="64" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="65" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="66" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="67" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="68" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="69" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="70" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="71" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="72" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="73" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="74" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="75" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="76" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="77" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="78" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="79" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="80" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="81" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="82" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="83" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="84" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="85" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="86" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="87" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="88" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="89" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="90" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="91" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="92" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="93" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="94" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="95" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="96" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="97" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="98" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="99" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="100" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="101" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="102" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="103" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="104" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="105" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="106" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="107" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="108" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="109" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="110" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="111" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="112" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="113" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="114" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="115" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="116" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="117" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="118" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="119" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="120" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="121" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="122" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="123" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="124" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="125" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="126" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="127" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="128" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="129" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="130" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="131" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="132" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="133" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="134" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="135" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="136" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="137" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="138" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="139" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="140" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="141" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="142" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="143" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="144" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="145" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="146" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="147" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="148" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="149" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="150" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="151" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="152" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="153" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="154" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="155" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="156" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="157" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="158" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="159" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="160" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="161" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="162" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="163" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="164" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="165" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="166" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="167" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="168" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="169" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="170" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="171" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="172" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="173" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="174" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="175" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="176" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="177" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="178" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="179" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="180" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="181" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="182" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="183" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="184" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="185" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="186" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="187" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="188" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="189" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="190" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="191" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="192" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="193" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="194" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="195" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="196" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="197" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="198" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="199" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="200" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="201" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="202" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="203" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="204" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="205" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="206" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="207" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="208" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="209" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="210" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="211" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="212" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="213" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="214" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="215" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="216" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="217" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="218" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="219" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="220" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="221" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="222" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="223" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="224" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="225" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="226" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="227" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="228" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="229" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="230" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="231" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="232" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="233" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="234" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="235" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="236" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="237" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="238" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="239" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="240" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="241" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="242" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="243" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="244" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="245" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="246" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="247" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="248" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="249" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="250" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="251" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="252" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="253" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="254" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="255" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="256" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="257" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="258" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="259" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="260" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="261" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="262" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="263" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="264" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="265" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="266" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="267" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="268" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="269" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="270" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="271" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="272" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="273" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="274" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="275" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="276" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="277" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="278" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="279" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="280" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="281" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="282" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="283" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="284" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="285" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="286" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="287" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="288" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="289" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="290" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="291" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="292" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="293" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="294" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="295" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="296" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="297" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="298" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="299" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="300" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="301" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="302" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="303" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="304" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="305" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="306" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="307" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="308" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="309" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="310" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="311" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="312" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="313" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="314" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="315" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="316" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="317" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="318" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="319" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="320" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="321" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="322" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="323" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="324" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="325" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="326" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="327" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="328" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="329" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="330" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="331" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="332" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="333" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="334" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="335" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="336" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="337" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="338" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="339" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="340" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="341" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="342" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="343" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="344" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="345" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="346" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="347" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="348" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="349" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="350" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="351" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="352" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="353" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="354" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="355" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="356" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="357" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="358" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="359" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="360" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="361" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="362" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="363" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="364" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="365" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="366" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="367" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="368" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="369" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="370" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="371" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="372" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="373" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="374" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="375" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="376" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="377" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="378" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="379" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="380" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="381" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="382" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="383" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="384" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="385" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="386" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="387" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="388" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="389" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="390" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="391" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="392" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="393" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="394" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="395" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="396" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="397" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="398" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="399" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="400" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="401" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="402" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="403" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="404" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="405" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="406" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="407" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="408" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="409" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="410" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="411" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="412" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="413" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="414" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="415" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="416" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="417" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="418" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="419" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="420" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="421" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="422" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="423" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="424" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="425" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="426" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="427" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="428" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="429" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="430" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="431" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="432" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="433" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="434" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="435" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="436" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="437" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="438" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="439" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="440" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="441" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="442" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="443" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="444" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="445" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="446" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="447" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="448" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="449" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="450" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="451" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="452" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="453" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="454" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="455" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="456" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="457" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="458" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="459" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="460" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="461" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="462" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="463" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="464" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="465" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="466" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="467" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="468" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="469" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="470" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="471" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="472" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="473" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="474" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="475" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="476" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="477" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="478" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="479" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="480" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="481" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="482" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="483" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="484" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="485" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="486" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="487" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="488" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="489" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="490" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="491" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="492" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="493" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="494" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="495" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="496" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="497" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="498" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="499" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="500" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="501" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="502" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="503" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="504" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="505" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="506" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="507" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="508" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="509" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="510" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="511" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="512" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="513" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="514" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="515" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="516" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="517" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="518" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="519" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="520" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="521" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="522" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="523" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="524" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="525" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="526" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="527" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="528" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="529" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="530" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="531" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="532" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="533" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="534" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="535" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="536" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="537" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="538" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="539" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="540" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="541" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="542" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="543" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="544" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="545" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="546" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="547" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="548" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="549" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="550" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="551" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="552" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="553" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="554" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="555" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="556" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="557" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="558" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="559" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="560" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="561" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="562" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="563" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="564" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="565" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="566" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="567" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="568" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="569" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="570" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="571" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="572" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="573" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="574" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="575" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="576" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="577" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="578" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="579" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="580" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="581" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="582" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="583" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="584" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="585" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="586" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="587" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="588" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="589" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="590" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="591" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="592" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="593" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="594" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="595" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="596" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="597" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="598" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="599" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="600" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="601" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="602" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="603" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="604" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="605" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="606" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="607" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="608" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="609" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="610" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="611" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="612" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="613" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="614" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="615" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="616" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="617" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="618" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="619" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="620" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="621" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="622" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="623" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="624" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="625" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="626" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="627" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="628" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="629" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="630" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="631" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="632" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="633" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="634" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="635" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="636" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="637" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="638" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="639" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="640" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="641" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="642" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="643" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="644" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="645" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="646" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="647" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="648" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="649" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="650" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="651" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="652" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="653" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="654" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="655" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="656" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="657" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="658" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="659" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="660" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="661" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="662" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="663" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="664" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="665" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="666" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="667" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="668" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="669" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="670" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="671" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="672" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="673" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="674" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="675" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="676" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="677" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="678" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="679" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="680" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="681" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="682" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="683" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="684" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="685" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="686" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="687" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="688" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="689" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="690" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="691" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="692" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="693" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="694" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="695" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="696" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="697" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="698" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="699" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="700" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="701" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="702" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="703" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="704" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="705" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="706" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="707" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="708" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="709" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="710" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="711" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="712" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="713" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="714" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="715" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="716" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="717" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="718" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="719" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="720" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="721" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="722" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="723" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="724" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="725" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="726" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="727" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="728" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="729" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="730" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="731" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="732" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="733" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="734" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="735" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="736" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="737" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="738" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="739" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="740" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="741" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="742" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="743" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="744" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="745" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="746" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="747" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="748" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="749" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="750" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="751" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="752" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="753" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="754" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="755" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="756" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="757" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="758" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="759" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="760" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="761" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="762" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="763" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="764" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="765" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="766" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="767" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="768" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="769" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="770" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="771" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="772" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="773" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="774" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="775" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="776" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="777" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="778" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="779" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="780" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="781" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="782" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="783" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="784" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="785" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="786" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="787" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="788" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="789" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="790" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="791" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="792" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="793" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="794" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="795" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="796" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="797" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="798" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="799" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="800" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="801" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="802" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="803" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="804" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="805" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="806" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="807" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="808" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="809" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="810" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="811" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="812" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="813" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="814" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="815" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="816" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="817" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="818" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="819" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="820" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="821" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="822" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="823" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="824" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="825" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="826" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="827" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="828" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="829" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="830" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="831" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="832" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="833" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="834" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="835" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="836" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="837" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="838" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="839" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="840" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="841" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="842" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="843" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="844" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="845" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="846" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="847" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="848" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="849" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="850" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="851" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="852" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="853" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="854" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="855" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="856" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="857" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="858" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="859" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="860" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="861" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="862" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="863" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="864" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="865" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="866" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="867" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="868" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="869" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="870" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="871" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="872" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="873" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="874" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="875" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="876" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="877" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="878" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="879" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="880" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="881" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="882" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="883" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="884" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="885" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="886" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="887" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="888" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="889" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="890" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="891" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="892" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="893" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="894" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="895" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="896" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="897" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="898" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="899" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="900" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="901" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="902" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="903" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="904" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="905" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="906" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="907" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="908" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="909" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="910" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="911" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="912" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="913" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="914" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="915" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="916" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="917" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="918" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="919" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="920" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="921" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="922" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="923" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="924" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="925" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="926" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="927" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="928" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="929" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="930" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="931" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="932" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="933" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="934" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="935" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="936" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="937" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="938" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="939" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="940" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="941" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="942" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="943" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="944" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="945" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="946" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="947" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="948" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="949" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="950" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="951" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="952" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="953" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="954" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="955" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="956" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="957" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="958" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="959" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="960" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="961" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="962" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="963" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="964" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="965" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="966" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="967" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="968" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="969" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="970" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="971" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="972" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="973" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="974" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="975" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="976" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="977" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="978" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="979" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="980" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="981" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="982" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="983" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="984" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="985" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="986" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="987" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="988" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="989" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="990" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="991" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="992" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="993" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="994" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="995" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="996" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="997" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="998" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="999" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="1000" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="49" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="50" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="51" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="52" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="53" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="54" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="55" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="56" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="57" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="58" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="59" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="60" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="61" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="62" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="63" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="64" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="65" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="66" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="67" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="68" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="69" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="70" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="71" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="72" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="73" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="74" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="75" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="76" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="77" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="78" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="79" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="80" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="81" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="82" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="83" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="84" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="85" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="86" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="87" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="88" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="89" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="90" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="91" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="92" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="93" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="94" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="95" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="96" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="97" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="98" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="99" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="100" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="101" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="102" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="103" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="104" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="105" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="106" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="107" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="108" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="109" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="110" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="111" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="112" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="113" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="114" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="115" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="116" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="117" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="118" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="119" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="120" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="121" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="122" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="123" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="124" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="125" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="126" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="127" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="128" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="129" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="130" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="131" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="132" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="133" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="134" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="135" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="136" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="137" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="138" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="139" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="140" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="141" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="142" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="143" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="144" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="145" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="146" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="147" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="148" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="149" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="150" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="151" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="152" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="153" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="154" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="155" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="156" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="157" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="158" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="159" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="160" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="161" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="162" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="163" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="164" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="165" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="166" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="167" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="168" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="169" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="170" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="171" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="172" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="173" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="174" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="175" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="176" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="177" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="178" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="179" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="180" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="181" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="182" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="183" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="184" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="185" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="186" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="187" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="188" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="189" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="190" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="191" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="192" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="193" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="194" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="195" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="196" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="197" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="198" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="199" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="200" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="201" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="202" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="203" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="204" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="205" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="206" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="207" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="208" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="209" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="210" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="211" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="212" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="213" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="214" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="215" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="216" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="217" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="218" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="219" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="220" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="221" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="222" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="223" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="224" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="225" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="226" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="227" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="228" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="229" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="230" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="231" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="232" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="233" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="234" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="235" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="236" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="237" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="238" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="239" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="240" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="241" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="242" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="243" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="244" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="245" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="246" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="247" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="248" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="249" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="250" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="251" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="252" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="253" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="254" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="255" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="256" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="257" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="258" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="259" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="260" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="261" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="262" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="263" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="264" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="265" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="266" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="267" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="268" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="269" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="270" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="271" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="272" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="273" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="274" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="275" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="276" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="277" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="278" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="279" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="280" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="281" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="282" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="283" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="284" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="285" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="286" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="287" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="288" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="289" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="290" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="291" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="292" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="293" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="294" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="295" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="296" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="297" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="298" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="299" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="300" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="301" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="302" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="303" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="304" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="305" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="306" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="307" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="308" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="309" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="310" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="311" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="312" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="313" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="314" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="315" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="316" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="317" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="318" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="319" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="320" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="321" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="322" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="323" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="324" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="325" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="326" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="327" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="328" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="329" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="330" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="331" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="332" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="333" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="334" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="335" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="336" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="337" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="338" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="339" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="340" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="341" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="342" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="343" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="344" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="345" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="346" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="347" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="348" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="349" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="350" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="351" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="352" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="353" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="354" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="355" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="356" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="357" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="358" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="359" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="360" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="361" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="362" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="363" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="364" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="365" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="366" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="367" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="368" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="369" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="370" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="371" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="372" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="373" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="374" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="375" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="376" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="377" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="378" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="379" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="380" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="381" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="382" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="383" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="384" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="385" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="386" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="387" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="388" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="389" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="390" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="391" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="392" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="393" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="394" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="395" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="396" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="397" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="398" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="399" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="400" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="401" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="402" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="403" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="404" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="405" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="406" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="407" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="408" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="409" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="410" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="411" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="412" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="413" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="414" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="415" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="416" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="417" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="418" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="419" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="420" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="421" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="422" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="423" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="424" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="425" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="426" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="427" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="428" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="429" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="430" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="431" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="432" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="433" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="434" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="435" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="436" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="437" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="438" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="439" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="440" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="441" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="442" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="443" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="444" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="445" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="446" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="447" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="448" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="449" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="450" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="451" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="452" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="453" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="454" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="455" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="456" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="457" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="458" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="459" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="460" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="461" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="462" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="463" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="464" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="465" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="466" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="467" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="468" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="469" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="470" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="471" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="472" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="473" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="474" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="475" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="476" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="477" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="478" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="479" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="480" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="481" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="482" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="483" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="484" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="485" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="486" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="487" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="488" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="489" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="490" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="491" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="492" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="493" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="494" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="495" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="496" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="497" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="498" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="499" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="500" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="501" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="502" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="503" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="504" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="505" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="506" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="507" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="508" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="509" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="510" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="511" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="512" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="513" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="514" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="515" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="516" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="517" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="518" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="519" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="520" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="521" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="522" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="523" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="524" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="525" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="526" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="527" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="528" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="529" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="530" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="531" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="532" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="533" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="534" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="535" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="536" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="537" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="538" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="539" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="540" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="541" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="542" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="543" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="544" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="545" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="546" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="547" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="548" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="549" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="550" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="551" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="552" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="553" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="554" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="555" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="556" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="557" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="558" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="559" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="560" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="561" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="562" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="563" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="564" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="565" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="566" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="567" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="568" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="569" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="570" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="571" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="572" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="573" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="574" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="575" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="576" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="577" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="578" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="579" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="580" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="581" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="582" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="583" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="584" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="585" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="586" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="587" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="588" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="589" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="590" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="591" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="592" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="593" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="594" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="595" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="596" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="597" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="598" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="599" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="600" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="601" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="602" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="603" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="604" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="605" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="606" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="607" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="608" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="609" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="610" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="611" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="612" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="613" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="614" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="615" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="616" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="617" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="618" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="619" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="620" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="621" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="622" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="623" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="624" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="625" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="626" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="627" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="628" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="629" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="630" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="631" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="632" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="633" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="634" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="635" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="636" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="637" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="638" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="639" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="640" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="641" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="642" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="643" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="644" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="645" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="646" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="647" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="648" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="649" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="650" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="651" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="652" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="653" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="654" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="655" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="656" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="657" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="658" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="659" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="660" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="661" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="662" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="663" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="664" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="665" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="666" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="667" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="668" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="669" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="670" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="671" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="672" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="673" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="674" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="675" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="676" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="677" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="678" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="679" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="680" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="681" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="682" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="683" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="684" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="685" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="686" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="687" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="688" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="689" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="690" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="691" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="692" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="693" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="694" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="695" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="696" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="697" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="698" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="699" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="700" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="701" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="702" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="703" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="704" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="705" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="706" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="707" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="708" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="709" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="710" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="711" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="712" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="713" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="714" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="715" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="716" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="717" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="718" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="719" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="720" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="721" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="722" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="723" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="724" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="725" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="726" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="727" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="728" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="729" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="730" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="731" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="732" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="733" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="734" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="735" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="736" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="737" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="738" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="739" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="740" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="741" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="742" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="743" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="744" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="745" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="746" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="747" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="748" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="749" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="750" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="751" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="752" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="753" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="754" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="755" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="756" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="757" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="758" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="759" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="760" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="761" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="762" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="763" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="764" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="765" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="766" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="767" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="768" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="769" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="770" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="771" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="772" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="773" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="774" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="775" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="776" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="777" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="778" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="779" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="780" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="781" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="782" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="783" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="784" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="785" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="786" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="787" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="788" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="789" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="790" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="791" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="792" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="793" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="794" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="795" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="796" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="797" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="798" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="799" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="800" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="801" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="802" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="803" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="804" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="805" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="806" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="807" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="808" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="809" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="810" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="811" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="812" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="813" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="814" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="815" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="816" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="817" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="818" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="819" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="820" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="821" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="822" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="823" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="824" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="825" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="826" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="827" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="828" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="829" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="830" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="831" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="832" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="833" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="834" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="835" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="836" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="837" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="838" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="839" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="840" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="841" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="842" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="843" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="844" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="845" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="846" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="847" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="848" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="849" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="850" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="851" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="852" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="853" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="854" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="855" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="856" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="857" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="858" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="859" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="860" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="861" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="862" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="863" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="864" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="865" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="866" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="867" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="868" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="869" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="870" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="871" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="872" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="873" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="874" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="875" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="876" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="877" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="878" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="879" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="880" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="881" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="882" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="883" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="884" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="885" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="886" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="887" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="888" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="889" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="890" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="891" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="892" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="893" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="894" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="895" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="896" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="897" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="898" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="899" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="900" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="901" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="902" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="903" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="904" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="905" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="906" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="907" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="908" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="909" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="910" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="911" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="912" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="913" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="914" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="915" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="916" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="917" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="918" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="919" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="920" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="921" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="922" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="923" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="924" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="925" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="926" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="927" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="928" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="929" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="930" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="931" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="932" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="933" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="934" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="935" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="936" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="937" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="938" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="939" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="940" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="941" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="942" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="943" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="944" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="945" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="946" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="947" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="948" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="949" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="950" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="951" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="952" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="953" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="954" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="955" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="956" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="957" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="958" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="959" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="960" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="961" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="962" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="963" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="964" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="965" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="966" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="967" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="968" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="969" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="970" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="971" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="972" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="973" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="974" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="975" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="976" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="977" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="978" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="979" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="980" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="981" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="982" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="983" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="984" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="985" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="986" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="987" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="988" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="989" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="990" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="991" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="992" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="993" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="994" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="995" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="996" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="997" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="998" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="999" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="1000" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
   </sheetData>
   <conditionalFormatting sqref="B2:Y45 Z2:AB44 AC2:AC45 AD2:AD44 AE2:AS45">
     <cfRule type="colorScale" priority="3">

</xml_diff>

<commit_message>
shortened name HERAMBIENTE termovalorizzatore
</commit_message>
<xml_diff>
--- a/southern_europe/italy_data/geographical_feature/node_metrics.xlsx
+++ b/southern_europe/italy_data/geographical_feature/node_metrics.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29127"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30131"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\0954659\PycharmProjects\AdOpT-NET0_luca\southern_europe\italy_data\geographical_feature\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E6818FCA-ECDD-428E-8F98-1F6452D13D4F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8846732B-F2FE-46E8-9A62-810990F3B6C3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="22932" yWindow="-6768" windowWidth="30936" windowHeight="16776" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="nodes" sheetId="1" r:id="rId1"/>
@@ -155,9 +155,6 @@
   </si>
   <si>
     <t>TERMOVALORIZZAOTRE DI VERONA</t>
-  </si>
-  <si>
-    <t>HERAMBIENTE S.R.L.  - IMPIANTO DI TERMOVALORIZZAZIONE RIFIUTI NON PERICOLOSI</t>
   </si>
   <si>
     <t>TERMOVALORIZZATORE DI BOLZANO</t>
@@ -534,6 +531,9 @@
   <si>
     <t>Piacenza</t>
   </si>
+  <si>
+    <t>HERAMBIENTE S.R.L.  - Termovalorizzatore</t>
+  </si>
 </sst>
 </file>
 
@@ -654,7 +654,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="24">
+  <cellXfs count="23">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="2" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
@@ -675,7 +675,6 @@
     <xf numFmtId="0" fontId="8" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="3" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="1"/>
@@ -898,7 +897,7 @@
   <sheetFormatPr defaultColWidth="11.09765625" defaultRowHeight="15" customHeight="1" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="10.5" customWidth="1"/>
-    <col min="2" max="2" width="39.5" customWidth="1"/>
+    <col min="2" max="2" width="72.3984375" customWidth="1"/>
     <col min="3" max="4" width="10.8984375" customWidth="1"/>
     <col min="5" max="5" width="10.5" customWidth="1"/>
     <col min="6" max="6" width="14.3984375" customWidth="1"/>
@@ -936,7 +935,7 @@
       <c r="A2" s="4">
         <v>1</v>
       </c>
-      <c r="B2" s="21" t="s">
+      <c r="B2" s="20" t="s">
         <v>8</v>
       </c>
       <c r="C2" s="2">
@@ -962,7 +961,7 @@
       <c r="A3" s="4">
         <v>2</v>
       </c>
-      <c r="B3" s="21" t="s">
+      <c r="B3" s="20" t="s">
         <v>10</v>
       </c>
       <c r="C3" s="2">
@@ -988,7 +987,7 @@
       <c r="A4" s="4">
         <v>3</v>
       </c>
-      <c r="B4" s="21" t="s">
+      <c r="B4" s="20" t="s">
         <v>12</v>
       </c>
       <c r="C4" s="5">
@@ -1014,7 +1013,7 @@
       <c r="A5" s="4">
         <v>4</v>
       </c>
-      <c r="B5" s="21" t="s">
+      <c r="B5" s="20" t="s">
         <v>14</v>
       </c>
       <c r="C5" s="2">
@@ -1040,7 +1039,7 @@
       <c r="A6" s="4">
         <v>5</v>
       </c>
-      <c r="B6" s="21" t="s">
+      <c r="B6" s="20" t="s">
         <v>15</v>
       </c>
       <c r="C6" s="2">
@@ -1066,7 +1065,7 @@
       <c r="A7" s="4">
         <v>6</v>
       </c>
-      <c r="B7" s="21" t="s">
+      <c r="B7" s="20" t="s">
         <v>16</v>
       </c>
       <c r="C7" s="2">
@@ -1092,7 +1091,7 @@
       <c r="A8" s="4">
         <v>7</v>
       </c>
-      <c r="B8" s="21" t="s">
+      <c r="B8" s="20" t="s">
         <v>17</v>
       </c>
       <c r="C8" s="2">
@@ -1118,7 +1117,7 @@
       <c r="A9" s="4">
         <v>8</v>
       </c>
-      <c r="B9" s="21" t="s">
+      <c r="B9" s="20" t="s">
         <v>19</v>
       </c>
       <c r="C9" s="2">
@@ -1144,7 +1143,7 @@
       <c r="A10" s="4">
         <v>9</v>
       </c>
-      <c r="B10" s="21" t="s">
+      <c r="B10" s="20" t="s">
         <v>20</v>
       </c>
       <c r="C10" s="2">
@@ -1170,7 +1169,7 @@
       <c r="A11" s="4">
         <v>10</v>
       </c>
-      <c r="B11" s="21" t="s">
+      <c r="B11" s="20" t="s">
         <v>21</v>
       </c>
       <c r="C11" s="2">
@@ -1196,7 +1195,7 @@
       <c r="A12" s="4">
         <v>11</v>
       </c>
-      <c r="B12" s="21" t="s">
+      <c r="B12" s="20" t="s">
         <v>22</v>
       </c>
       <c r="C12" s="2">
@@ -1222,7 +1221,7 @@
       <c r="A13" s="4">
         <v>12</v>
       </c>
-      <c r="B13" s="21" t="s">
+      <c r="B13" s="20" t="s">
         <v>23</v>
       </c>
       <c r="C13" s="2">
@@ -1248,7 +1247,7 @@
       <c r="A14" s="4">
         <v>13</v>
       </c>
-      <c r="B14" s="21" t="s">
+      <c r="B14" s="20" t="s">
         <v>24</v>
       </c>
       <c r="C14" s="2">
@@ -1274,7 +1273,7 @@
       <c r="A15" s="4">
         <v>14</v>
       </c>
-      <c r="B15" s="21" t="s">
+      <c r="B15" s="20" t="s">
         <v>25</v>
       </c>
       <c r="C15" s="2">
@@ -1300,7 +1299,7 @@
       <c r="A16" s="4">
         <v>15</v>
       </c>
-      <c r="B16" s="21" t="s">
+      <c r="B16" s="20" t="s">
         <v>26</v>
       </c>
       <c r="C16" s="2">
@@ -1326,7 +1325,7 @@
       <c r="A17" s="4">
         <v>16</v>
       </c>
-      <c r="B17" s="21" t="s">
+      <c r="B17" s="20" t="s">
         <v>27</v>
       </c>
       <c r="C17" s="2">
@@ -1352,7 +1351,7 @@
       <c r="A18" s="4">
         <v>17</v>
       </c>
-      <c r="B18" s="21" t="s">
+      <c r="B18" s="20" t="s">
         <v>28</v>
       </c>
       <c r="C18" s="2">
@@ -1378,7 +1377,7 @@
       <c r="A19" s="4">
         <v>18</v>
       </c>
-      <c r="B19" s="21" t="s">
+      <c r="B19" s="20" t="s">
         <v>29</v>
       </c>
       <c r="C19" s="2">
@@ -1404,7 +1403,7 @@
       <c r="A20" s="4">
         <v>19</v>
       </c>
-      <c r="B20" s="21" t="s">
+      <c r="B20" s="20" t="s">
         <v>30</v>
       </c>
       <c r="C20" s="2">
@@ -1430,8 +1429,8 @@
       <c r="A21" s="4">
         <v>20</v>
       </c>
-      <c r="B21" s="21" t="s">
-        <v>162</v>
+      <c r="B21" s="20" t="s">
+        <v>161</v>
       </c>
       <c r="C21" s="2">
         <v>9.7038200000000003</v>
@@ -1456,8 +1455,8 @@
       <c r="A22" s="4">
         <v>20</v>
       </c>
-      <c r="B22" s="21" t="s">
-        <v>162</v>
+      <c r="B22" s="20" t="s">
+        <v>161</v>
       </c>
       <c r="C22" s="2">
         <v>9.7038200000000003</v>
@@ -1482,7 +1481,7 @@
       <c r="A23" s="4">
         <v>21</v>
       </c>
-      <c r="B23" s="21" t="s">
+      <c r="B23" s="20" t="s">
         <v>31</v>
       </c>
       <c r="C23" s="2">
@@ -1508,7 +1507,7 @@
       <c r="A24" s="4">
         <v>22</v>
       </c>
-      <c r="B24" s="21" t="s">
+      <c r="B24" s="20" t="s">
         <v>32</v>
       </c>
       <c r="C24" s="2">
@@ -1534,7 +1533,7 @@
       <c r="A25" s="4">
         <v>23</v>
       </c>
-      <c r="B25" s="21" t="s">
+      <c r="B25" s="20" t="s">
         <v>33</v>
       </c>
       <c r="C25" s="2">
@@ -1560,7 +1559,7 @@
       <c r="A26" s="4">
         <v>24</v>
       </c>
-      <c r="B26" s="21" t="s">
+      <c r="B26" s="20" t="s">
         <v>34</v>
       </c>
       <c r="C26" s="2">
@@ -1586,7 +1585,7 @@
       <c r="A27" s="4">
         <v>25</v>
       </c>
-      <c r="B27" s="21" t="s">
+      <c r="B27" s="20" t="s">
         <v>35</v>
       </c>
       <c r="C27" s="2">
@@ -1612,7 +1611,7 @@
       <c r="A28" s="4">
         <v>26</v>
       </c>
-      <c r="B28" s="21" t="s">
+      <c r="B28" s="20" t="s">
         <v>36</v>
       </c>
       <c r="C28" s="2">
@@ -1638,8 +1637,8 @@
       <c r="A29" s="4">
         <v>27</v>
       </c>
-      <c r="B29" s="21" t="s">
-        <v>37</v>
+      <c r="B29" s="20" t="s">
+        <v>162</v>
       </c>
       <c r="C29" s="2">
         <v>10.943759999999999</v>
@@ -1664,8 +1663,8 @@
       <c r="A30" s="4">
         <v>28</v>
       </c>
-      <c r="B30" s="21" t="s">
-        <v>38</v>
+      <c r="B30" s="20" t="s">
+        <v>37</v>
       </c>
       <c r="C30" s="2">
         <v>11.30925</v>
@@ -1690,8 +1689,8 @@
       <c r="A31" s="4">
         <v>29</v>
       </c>
-      <c r="B31" s="21" t="s">
-        <v>39</v>
+      <c r="B31" s="20" t="s">
+        <v>38</v>
       </c>
       <c r="C31" s="2">
         <v>11.556369999999999</v>
@@ -1716,8 +1715,8 @@
       <c r="A32" s="4">
         <v>30</v>
       </c>
-      <c r="B32" s="21" t="s">
-        <v>40</v>
+      <c r="B32" s="20" t="s">
+        <v>39</v>
       </c>
       <c r="C32" s="2">
         <v>11.428890000000001</v>
@@ -1742,8 +1741,8 @@
       <c r="A33" s="4">
         <v>31</v>
       </c>
-      <c r="B33" s="21" t="s">
-        <v>41</v>
+      <c r="B33" s="20" t="s">
+        <v>40</v>
       </c>
       <c r="C33" s="2">
         <v>11.75079</v>
@@ -1768,8 +1767,8 @@
       <c r="A34" s="4">
         <v>32</v>
       </c>
-      <c r="B34" s="21" t="s">
-        <v>42</v>
+      <c r="B34" s="20" t="s">
+        <v>41</v>
       </c>
       <c r="C34" s="5">
         <v>11.69642</v>
@@ -1794,8 +1793,8 @@
       <c r="A35" s="4">
         <v>33</v>
       </c>
-      <c r="B35" s="21" t="s">
-        <v>43</v>
+      <c r="B35" s="20" t="s">
+        <v>42</v>
       </c>
       <c r="C35" s="2">
         <v>11.963570000000001</v>
@@ -1820,8 +1819,8 @@
       <c r="A36" s="4">
         <v>34</v>
       </c>
-      <c r="B36" s="21" t="s">
-        <v>44</v>
+      <c r="B36" s="20" t="s">
+        <v>43</v>
       </c>
       <c r="C36" s="2">
         <v>11.924099999999999</v>
@@ -1846,8 +1845,8 @@
       <c r="A37" s="4">
         <v>35</v>
       </c>
-      <c r="B37" s="21" t="s">
-        <v>45</v>
+      <c r="B37" s="20" t="s">
+        <v>44</v>
       </c>
       <c r="C37" s="2">
         <v>12.08798</v>
@@ -1872,8 +1871,8 @@
       <c r="A38" s="4">
         <v>36</v>
       </c>
-      <c r="B38" s="21" t="s">
-        <v>46</v>
+      <c r="B38" s="20" t="s">
+        <v>45</v>
       </c>
       <c r="C38" s="2">
         <v>12.269209999999999</v>
@@ -1898,8 +1897,8 @@
       <c r="A39" s="4">
         <v>37</v>
       </c>
-      <c r="B39" s="21" t="s">
-        <v>47</v>
+      <c r="B39" s="20" t="s">
+        <v>46</v>
       </c>
       <c r="C39" s="2">
         <v>12.2</v>
@@ -1917,15 +1916,15 @@
         <v>0</v>
       </c>
       <c r="H39" s="1" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
     </row>
     <row r="40" spans="1:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A40" s="4">
         <v>38</v>
       </c>
-      <c r="B40" s="21" t="s">
-        <v>49</v>
+      <c r="B40" s="20" t="s">
+        <v>48</v>
       </c>
       <c r="C40" s="5">
         <v>12.31551</v>
@@ -1950,8 +1949,8 @@
       <c r="A41" s="4">
         <v>39</v>
       </c>
-      <c r="B41" s="21" t="s">
-        <v>50</v>
+      <c r="B41" s="20" t="s">
+        <v>49</v>
       </c>
       <c r="C41" s="2">
         <v>12.74245</v>
@@ -1976,8 +1975,8 @@
       <c r="A42" s="4">
         <v>40</v>
       </c>
-      <c r="B42" s="21" t="s">
-        <v>51</v>
+      <c r="B42" s="20" t="s">
+        <v>50</v>
       </c>
       <c r="C42" s="2">
         <v>12.63189</v>
@@ -2002,8 +2001,8 @@
       <c r="A43" s="4">
         <v>41</v>
       </c>
-      <c r="B43" s="21" t="s">
-        <v>52</v>
+      <c r="B43" s="20" t="s">
+        <v>51</v>
       </c>
       <c r="C43" s="2">
         <v>13.80006</v>
@@ -2028,8 +2027,8 @@
       <c r="A44" s="4">
         <v>42</v>
       </c>
-      <c r="B44" s="21" t="s">
-        <v>160</v>
+      <c r="B44" s="20" t="s">
+        <v>159</v>
       </c>
       <c r="C44" s="2">
         <v>12.274480000000001</v>
@@ -2054,8 +2053,8 @@
       <c r="A45" s="4">
         <v>43</v>
       </c>
-      <c r="B45" s="21" t="s">
-        <v>53</v>
+      <c r="B45" s="20" t="s">
+        <v>52</v>
       </c>
       <c r="C45" s="5">
         <v>12.564</v>
@@ -2073,7 +2072,7 @@
         <v>0</v>
       </c>
       <c r="H45" s="1" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
     </row>
     <row r="46" spans="1:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
@@ -2081,7 +2080,7 @@
         <v>44</v>
       </c>
       <c r="B46" s="4" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="C46" s="4">
         <v>10.64</v>
@@ -6063,7 +6062,7 @@
       <c r="AR1" s="4">
         <v>43</v>
       </c>
-      <c r="AS1" s="20">
+      <c r="AS1">
         <v>44</v>
       </c>
     </row>
@@ -11956,7 +11955,7 @@
       </c>
     </row>
     <row r="45" spans="1:45" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A45" s="20">
+      <c r="A45">
         <v>44</v>
       </c>
       <c r="B45" s="4">
@@ -27345,7 +27344,7 @@
   <dimension ref="A1:Z1000"/>
   <sheetFormatPr defaultColWidth="11.09765625" defaultRowHeight="15" customHeight="1" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="41.5" customWidth="1"/>
+    <col min="1" max="1" width="88.09765625" customWidth="1"/>
     <col min="2" max="3" width="11" customWidth="1"/>
     <col min="4" max="4" width="14.5" customWidth="1"/>
     <col min="5" max="8" width="10.5" customWidth="1"/>
@@ -27357,45 +27356,45 @@
   <sheetData>
     <row r="1" spans="1:26" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A1" s="12" t="s">
+        <v>55</v>
+      </c>
+      <c r="B1" s="13" t="s">
         <v>56</v>
       </c>
-      <c r="B1" s="13" t="s">
+      <c r="C1" s="13" t="s">
         <v>57</v>
       </c>
-      <c r="C1" s="13" t="s">
+      <c r="D1" s="12" t="s">
         <v>58</v>
       </c>
-      <c r="D1" s="12" t="s">
+      <c r="E1" s="12" t="s">
         <v>59</v>
       </c>
-      <c r="E1" s="12" t="s">
+      <c r="F1" s="12" t="s">
         <v>60</v>
       </c>
-      <c r="F1" s="12" t="s">
+      <c r="G1" s="12" t="s">
         <v>61</v>
       </c>
-      <c r="G1" s="12" t="s">
+      <c r="H1" s="12" t="s">
         <v>62</v>
       </c>
-      <c r="H1" s="12" t="s">
+      <c r="I1" s="12" t="s">
         <v>63</v>
       </c>
-      <c r="I1" s="12" t="s">
+      <c r="J1" s="12" t="s">
         <v>64</v>
       </c>
-      <c r="J1" s="12" t="s">
+      <c r="K1" s="12" t="s">
         <v>65</v>
       </c>
-      <c r="K1" s="12" t="s">
+      <c r="L1" s="12" t="s">
         <v>66</v>
-      </c>
-      <c r="L1" s="12" t="s">
-        <v>67</v>
       </c>
     </row>
     <row r="2" spans="1:26" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A2" s="14" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="B2" s="15">
         <v>11.75079</v>
@@ -27410,25 +27409,25 @@
         <v>11</v>
       </c>
       <c r="F2" s="14" t="s">
+        <v>67</v>
+      </c>
+      <c r="G2" s="14" t="s">
         <v>68</v>
       </c>
-      <c r="G2" s="14" t="s">
+      <c r="H2" s="14" t="s">
         <v>69</v>
-      </c>
-      <c r="H2" s="14" t="s">
-        <v>70</v>
       </c>
       <c r="I2" s="14">
         <v>800000</v>
       </c>
       <c r="J2" s="14" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="K2" s="14">
         <v>2021</v>
       </c>
       <c r="L2" s="17" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="M2" s="18"/>
       <c r="N2" s="18"/>
@@ -27447,7 +27446,7 @@
     </row>
     <row r="3" spans="1:26" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A3" s="14" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="B3" s="15">
         <v>11.963570000000001</v>
@@ -27462,13 +27461,13 @@
         <v>11</v>
       </c>
       <c r="F3" s="14" t="s">
+        <v>72</v>
+      </c>
+      <c r="G3" s="14" t="s">
         <v>73</v>
       </c>
-      <c r="G3" s="14" t="s">
+      <c r="H3" s="14" t="s">
         <v>74</v>
-      </c>
-      <c r="H3" s="14" t="s">
-        <v>75</v>
       </c>
       <c r="I3" s="14">
         <v>1000000</v>
@@ -27478,7 +27477,7 @@
         <v>2021</v>
       </c>
       <c r="L3" s="17" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="M3" s="18"/>
       <c r="N3" s="18"/>
@@ -27497,7 +27496,7 @@
     </row>
     <row r="4" spans="1:26" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A4" s="14" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="B4" s="15">
         <v>12.269209999999999</v>
@@ -27512,23 +27511,23 @@
         <v>11</v>
       </c>
       <c r="F4" s="14" t="s">
+        <v>75</v>
+      </c>
+      <c r="G4" s="14" t="s">
+        <v>73</v>
+      </c>
+      <c r="H4" s="14" t="s">
         <v>76</v>
       </c>
-      <c r="G4" s="14" t="s">
-        <v>74</v>
-      </c>
-      <c r="H4" s="14" t="s">
+      <c r="I4" s="14" t="s">
         <v>77</v>
-      </c>
-      <c r="I4" s="14" t="s">
-        <v>78</v>
       </c>
       <c r="J4" s="14"/>
       <c r="K4" s="14">
         <v>2021</v>
       </c>
       <c r="L4" s="17" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="M4" s="18"/>
       <c r="N4" s="18"/>
@@ -27562,25 +27561,25 @@
         <v>11</v>
       </c>
       <c r="F5" s="14" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="G5" s="14" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="H5" s="14" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="I5" s="14">
         <v>1600000</v>
       </c>
       <c r="J5" s="14" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="K5" s="14">
         <v>2021</v>
       </c>
       <c r="L5" s="17" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="M5" s="18"/>
       <c r="N5" s="18"/>
@@ -27614,13 +27613,13 @@
         <v>11</v>
       </c>
       <c r="F6" s="14" t="s">
+        <v>79</v>
+      </c>
+      <c r="G6" s="14" t="s">
         <v>80</v>
       </c>
-      <c r="G6" s="14" t="s">
+      <c r="H6" s="14" t="s">
         <v>81</v>
-      </c>
-      <c r="H6" s="14" t="s">
-        <v>82</v>
       </c>
       <c r="I6" s="14"/>
       <c r="J6" s="14"/>
@@ -27628,7 +27627,7 @@
         <v>2021</v>
       </c>
       <c r="L6" s="17" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="M6" s="18"/>
       <c r="N6" s="18"/>
@@ -27662,25 +27661,25 @@
         <v>11</v>
       </c>
       <c r="F7" s="14" t="s">
+        <v>82</v>
+      </c>
+      <c r="G7" s="14" t="s">
+        <v>73</v>
+      </c>
+      <c r="H7" s="14" t="s">
         <v>83</v>
-      </c>
-      <c r="G7" s="14" t="s">
-        <v>74</v>
-      </c>
-      <c r="H7" s="14" t="s">
-        <v>84</v>
       </c>
       <c r="I7" s="14">
         <v>1500000</v>
       </c>
       <c r="J7" s="14" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="K7" s="14">
         <v>2021</v>
       </c>
       <c r="L7" s="17" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="M7" s="18"/>
       <c r="N7" s="18"/>
@@ -27714,21 +27713,21 @@
         <v>11</v>
       </c>
       <c r="F8" s="14" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="G8" s="14"/>
       <c r="H8" s="14" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="I8" s="14" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="J8" s="14"/>
       <c r="K8" s="14">
         <v>2021</v>
       </c>
       <c r="L8" s="17" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="M8" s="18"/>
       <c r="N8" s="18"/>
@@ -27762,25 +27761,25 @@
         <v>11</v>
       </c>
       <c r="F9" s="14" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="G9" s="14" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="H9" s="14" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="I9" s="14">
         <v>1300000</v>
       </c>
       <c r="J9" s="14" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="K9" s="14">
         <v>2021</v>
       </c>
       <c r="L9" s="17" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="M9" s="18"/>
       <c r="N9" s="18"/>
@@ -27814,23 +27813,23 @@
         <v>11</v>
       </c>
       <c r="F10" s="14" t="s">
+        <v>87</v>
+      </c>
+      <c r="G10" s="14" t="s">
+        <v>73</v>
+      </c>
+      <c r="H10" s="14" t="s">
         <v>88</v>
       </c>
-      <c r="G10" s="14" t="s">
-        <v>74</v>
-      </c>
-      <c r="H10" s="14" t="s">
-        <v>89</v>
-      </c>
       <c r="I10" s="14" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="J10" s="14"/>
       <c r="K10" s="14">
         <v>2021</v>
       </c>
       <c r="L10" s="17" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="M10" s="18"/>
       <c r="N10" s="18"/>
@@ -27864,23 +27863,23 @@
         <v>11</v>
       </c>
       <c r="F11" s="14" t="s">
+        <v>89</v>
+      </c>
+      <c r="G11" s="14" t="s">
+        <v>73</v>
+      </c>
+      <c r="H11" s="14" t="s">
         <v>90</v>
       </c>
-      <c r="G11" s="14" t="s">
-        <v>74</v>
-      </c>
-      <c r="H11" s="14" t="s">
-        <v>91</v>
-      </c>
       <c r="I11" s="14" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="J11" s="14"/>
       <c r="K11" s="14">
         <v>2021</v>
       </c>
       <c r="L11" s="17" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="M11" s="18"/>
       <c r="N11" s="18"/>
@@ -27899,7 +27898,7 @@
     </row>
     <row r="12" spans="1:26" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A12" s="14" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="B12" s="15">
         <v>12.74245</v>
@@ -27914,25 +27913,25 @@
         <v>11</v>
       </c>
       <c r="F12" s="14" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="G12" s="14" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="H12" s="14" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
       <c r="I12" s="14">
         <v>1000000</v>
       </c>
       <c r="J12" s="14" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="K12" s="14">
         <v>2021</v>
       </c>
       <c r="L12" s="17" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="M12" s="18"/>
       <c r="N12" s="18"/>
@@ -27951,7 +27950,7 @@
     </row>
     <row r="13" spans="1:26" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A13" s="14" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="B13" s="15">
         <v>9.7164300000000008</v>
@@ -27966,13 +27965,13 @@
         <v>11</v>
       </c>
       <c r="F13" s="14" t="s">
+        <v>72</v>
+      </c>
+      <c r="G13" s="14" t="s">
         <v>73</v>
       </c>
-      <c r="G13" s="14" t="s">
-        <v>74</v>
-      </c>
       <c r="H13" s="14" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
       <c r="I13" s="14">
         <v>1000000</v>
@@ -27982,7 +27981,7 @@
         <v>2021</v>
       </c>
       <c r="L13" s="17" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="M13" s="18"/>
       <c r="N13" s="18"/>
@@ -28016,25 +28015,25 @@
         <v>11</v>
       </c>
       <c r="F14" s="14" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="G14" s="14" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="H14" s="14" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
       <c r="I14" s="14">
         <v>1300000</v>
       </c>
       <c r="J14" s="14" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="K14" s="14">
         <v>2021</v>
       </c>
       <c r="L14" s="17" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="M14" s="18"/>
       <c r="N14" s="18"/>
@@ -28069,10 +28068,10 @@
       </c>
       <c r="F15" s="14"/>
       <c r="G15" s="14" t="s">
+        <v>95</v>
+      </c>
+      <c r="H15" s="14" t="s">
         <v>96</v>
-      </c>
-      <c r="H15" s="14" t="s">
-        <v>97</v>
       </c>
       <c r="I15" s="14"/>
       <c r="J15" s="14"/>
@@ -28080,7 +28079,7 @@
         <v>2021</v>
       </c>
       <c r="L15" s="17" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="M15" s="18"/>
       <c r="N15" s="18"/>
@@ -28114,13 +28113,13 @@
         <v>18</v>
       </c>
       <c r="F16" s="14" t="s">
+        <v>97</v>
+      </c>
+      <c r="G16" s="14" t="s">
+        <v>95</v>
+      </c>
+      <c r="H16" s="14" t="s">
         <v>98</v>
-      </c>
-      <c r="G16" s="14" t="s">
-        <v>96</v>
-      </c>
-      <c r="H16" s="14" t="s">
-        <v>99</v>
       </c>
       <c r="I16" s="14"/>
       <c r="J16" s="14"/>
@@ -28128,7 +28127,7 @@
         <v>2021</v>
       </c>
       <c r="L16" s="17" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="M16" s="18"/>
       <c r="N16" s="18"/>
@@ -28162,13 +28161,13 @@
         <v>18</v>
       </c>
       <c r="F17" s="14" t="s">
+        <v>99</v>
+      </c>
+      <c r="G17" s="14" t="s">
+        <v>95</v>
+      </c>
+      <c r="H17" s="14" t="s">
         <v>100</v>
-      </c>
-      <c r="G17" s="14" t="s">
-        <v>96</v>
-      </c>
-      <c r="H17" s="14" t="s">
-        <v>101</v>
       </c>
       <c r="I17" s="14"/>
       <c r="J17" s="14"/>
@@ -28176,7 +28175,7 @@
         <v>2021</v>
       </c>
       <c r="L17" s="17" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="M17" s="18"/>
       <c r="N17" s="18"/>
@@ -28195,7 +28194,7 @@
     </row>
     <row r="18" spans="1:26" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A18" s="14" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="B18" s="15">
         <v>11.924099999999999</v>
@@ -28210,25 +28209,25 @@
         <v>9</v>
       </c>
       <c r="F18" s="14" t="s">
+        <v>101</v>
+      </c>
+      <c r="G18" s="14" t="s">
         <v>102</v>
       </c>
-      <c r="G18" s="14" t="s">
+      <c r="H18" s="14" t="s">
         <v>103</v>
-      </c>
-      <c r="H18" s="14" t="s">
-        <v>104</v>
       </c>
       <c r="I18" s="14">
         <v>600</v>
       </c>
       <c r="J18" s="14" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
       <c r="K18" s="14">
         <v>2021</v>
       </c>
       <c r="L18" s="17" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="M18" s="18"/>
       <c r="N18" s="18"/>
@@ -28262,25 +28261,25 @@
         <v>9</v>
       </c>
       <c r="F19" s="14" t="s">
+        <v>105</v>
+      </c>
+      <c r="G19" s="14" t="s">
+        <v>102</v>
+      </c>
+      <c r="H19" s="14" t="s">
         <v>106</v>
-      </c>
-      <c r="G19" s="14" t="s">
-        <v>103</v>
-      </c>
-      <c r="H19" s="14" t="s">
-        <v>107</v>
       </c>
       <c r="I19" s="14">
         <v>180000</v>
       </c>
       <c r="J19" s="14" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="K19" s="14" t="s">
+        <v>107</v>
+      </c>
+      <c r="L19" s="14" t="s">
         <v>108</v>
-      </c>
-      <c r="L19" s="14" t="s">
-        <v>109</v>
       </c>
       <c r="M19" s="18"/>
       <c r="N19" s="18"/>
@@ -28299,7 +28298,7 @@
     </row>
     <row r="20" spans="1:26" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A20" s="14" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="B20" s="15">
         <v>11.30925</v>
@@ -28314,25 +28313,25 @@
         <v>9</v>
       </c>
       <c r="F20" s="14" t="s">
+        <v>109</v>
+      </c>
+      <c r="G20" s="14" t="s">
+        <v>102</v>
+      </c>
+      <c r="H20" s="14" t="s">
         <v>110</v>
-      </c>
-      <c r="G20" s="14" t="s">
-        <v>103</v>
-      </c>
-      <c r="H20" s="14" t="s">
-        <v>111</v>
       </c>
       <c r="I20" s="14">
         <v>130000</v>
       </c>
       <c r="J20" s="14" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="K20" s="14" t="s">
+        <v>107</v>
+      </c>
+      <c r="L20" s="14" t="s">
         <v>108</v>
-      </c>
-      <c r="L20" s="14" t="s">
-        <v>109</v>
       </c>
       <c r="M20" s="18"/>
       <c r="N20" s="18"/>
@@ -28366,25 +28365,25 @@
         <v>9</v>
       </c>
       <c r="F21" s="14" t="s">
+        <v>111</v>
+      </c>
+      <c r="G21" s="14" t="s">
+        <v>102</v>
+      </c>
+      <c r="H21" s="14" t="s">
         <v>112</v>
-      </c>
-      <c r="G21" s="14" t="s">
-        <v>103</v>
-      </c>
-      <c r="H21" s="14" t="s">
-        <v>113</v>
       </c>
       <c r="I21" s="14">
         <v>421000</v>
       </c>
       <c r="J21" s="14" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="K21" s="14">
         <v>2021</v>
       </c>
       <c r="L21" s="17" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="M21" s="18"/>
       <c r="N21" s="18"/>
@@ -28418,25 +28417,25 @@
         <v>9</v>
       </c>
       <c r="F22" s="14" t="s">
+        <v>113</v>
+      </c>
+      <c r="G22" s="14" t="s">
+        <v>102</v>
+      </c>
+      <c r="H22" s="14" t="s">
         <v>114</v>
-      </c>
-      <c r="G22" s="14" t="s">
-        <v>103</v>
-      </c>
-      <c r="H22" s="14" t="s">
-        <v>115</v>
       </c>
       <c r="I22" s="14">
         <v>730000</v>
       </c>
       <c r="J22" s="14" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="K22" s="14">
         <v>2022</v>
       </c>
       <c r="L22" s="14" t="s">
-        <v>116</v>
+        <v>115</v>
       </c>
       <c r="M22" s="18"/>
       <c r="N22" s="18"/>
@@ -28470,25 +28469,25 @@
         <v>9</v>
       </c>
       <c r="F23" s="14" t="s">
+        <v>116</v>
+      </c>
+      <c r="G23" s="14" t="s">
+        <v>102</v>
+      </c>
+      <c r="H23" s="14" t="s">
         <v>117</v>
-      </c>
-      <c r="G23" s="14" t="s">
-        <v>103</v>
-      </c>
-      <c r="H23" s="14" t="s">
-        <v>118</v>
       </c>
       <c r="I23" s="14">
         <v>110000</v>
       </c>
       <c r="J23" s="14" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="K23" s="14" t="s">
+        <v>107</v>
+      </c>
+      <c r="L23" s="14" t="s">
         <v>108</v>
-      </c>
-      <c r="L23" s="14" t="s">
-        <v>109</v>
       </c>
       <c r="M23" s="18"/>
       <c r="N23" s="18"/>
@@ -28522,25 +28521,25 @@
         <v>9</v>
       </c>
       <c r="F24" s="14" t="s">
+        <v>118</v>
+      </c>
+      <c r="G24" s="14" t="s">
+        <v>102</v>
+      </c>
+      <c r="H24" s="14" t="s">
         <v>119</v>
-      </c>
-      <c r="G24" s="14" t="s">
-        <v>103</v>
-      </c>
-      <c r="H24" s="14" t="s">
-        <v>120</v>
       </c>
       <c r="I24" s="14">
         <v>93000</v>
       </c>
       <c r="J24" s="14" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="K24" s="14">
         <v>2021</v>
       </c>
       <c r="L24" s="17" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="M24" s="18"/>
       <c r="N24" s="18"/>
@@ -28574,25 +28573,25 @@
         <v>9</v>
       </c>
       <c r="F25" s="14" t="s">
+        <v>120</v>
+      </c>
+      <c r="G25" s="14" t="s">
+        <v>102</v>
+      </c>
+      <c r="H25" s="14" t="s">
         <v>121</v>
-      </c>
-      <c r="G25" s="14" t="s">
-        <v>103</v>
-      </c>
-      <c r="H25" s="14" t="s">
-        <v>122</v>
       </c>
       <c r="I25" s="14">
         <v>150000</v>
       </c>
       <c r="J25" s="14" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="K25" s="14">
         <v>2021</v>
       </c>
       <c r="L25" s="17" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="M25" s="18"/>
       <c r="N25" s="18"/>
@@ -28626,25 +28625,25 @@
         <v>9</v>
       </c>
       <c r="F26" s="14" t="s">
+        <v>122</v>
+      </c>
+      <c r="G26" s="14" t="s">
+        <v>102</v>
+      </c>
+      <c r="H26" s="14" t="s">
         <v>123</v>
-      </c>
-      <c r="G26" s="14" t="s">
-        <v>103</v>
-      </c>
-      <c r="H26" s="14" t="s">
-        <v>124</v>
       </c>
       <c r="I26" s="14">
         <v>100000</v>
       </c>
       <c r="J26" s="14" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="K26" s="14" t="s">
+        <v>107</v>
+      </c>
+      <c r="L26" s="14" t="s">
         <v>108</v>
-      </c>
-      <c r="L26" s="14" t="s">
-        <v>109</v>
       </c>
       <c r="M26" s="18"/>
       <c r="N26" s="18"/>
@@ -28678,25 +28677,25 @@
         <v>9</v>
       </c>
       <c r="F27" s="14" t="s">
-        <v>114</v>
+        <v>113</v>
       </c>
       <c r="G27" s="14" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="H27" s="14" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="I27" s="14">
         <v>540000</v>
       </c>
       <c r="J27" s="14" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="K27" s="14">
         <v>2021</v>
       </c>
       <c r="L27" s="17" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="M27" s="18"/>
       <c r="N27" s="18"/>
@@ -28730,25 +28729,25 @@
         <v>9</v>
       </c>
       <c r="F28" s="14" t="s">
-        <v>114</v>
+        <v>113</v>
       </c>
       <c r="G28" s="14" t="s">
+        <v>125</v>
+      </c>
+      <c r="H28" s="14" t="s">
         <v>126</v>
-      </c>
-      <c r="H28" s="14" t="s">
-        <v>127</v>
       </c>
       <c r="I28" s="14">
         <v>160000</v>
       </c>
       <c r="J28" s="14" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="K28" s="14" t="s">
+        <v>107</v>
+      </c>
+      <c r="L28" s="14" t="s">
         <v>108</v>
-      </c>
-      <c r="L28" s="14" t="s">
-        <v>109</v>
       </c>
       <c r="M28" s="18"/>
       <c r="N28" s="18"/>
@@ -28782,25 +28781,25 @@
         <v>9</v>
       </c>
       <c r="F29" s="14" t="s">
+        <v>127</v>
+      </c>
+      <c r="G29" s="14" t="s">
+        <v>102</v>
+      </c>
+      <c r="H29" s="14" t="s">
         <v>128</v>
-      </c>
-      <c r="G29" s="14" t="s">
-        <v>103</v>
-      </c>
-      <c r="H29" s="14" t="s">
-        <v>129</v>
       </c>
       <c r="I29" s="14">
         <v>174900</v>
       </c>
       <c r="J29" s="14" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="K29" s="14">
         <v>2021</v>
       </c>
       <c r="L29" s="17" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="M29" s="18"/>
       <c r="N29" s="18"/>
@@ -28834,25 +28833,25 @@
         <v>9</v>
       </c>
       <c r="F30" s="14" t="s">
+        <v>129</v>
+      </c>
+      <c r="G30" s="14" t="s">
+        <v>102</v>
+      </c>
+      <c r="H30" s="14" t="s">
         <v>130</v>
-      </c>
-      <c r="G30" s="14" t="s">
-        <v>103</v>
-      </c>
-      <c r="H30" s="14" t="s">
-        <v>131</v>
       </c>
       <c r="I30" s="14">
         <v>93400</v>
       </c>
       <c r="J30" s="14" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="K30" s="14">
         <v>2021</v>
       </c>
       <c r="L30" s="17" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="M30" s="18"/>
       <c r="N30" s="18"/>
@@ -28871,7 +28870,7 @@
     </row>
     <row r="31" spans="1:26" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A31" s="14" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="B31" s="15">
         <v>13.80006</v>
@@ -28886,25 +28885,25 @@
         <v>9</v>
       </c>
       <c r="F31" s="14" t="s">
+        <v>101</v>
+      </c>
+      <c r="G31" s="14" t="s">
         <v>102</v>
       </c>
-      <c r="G31" s="14" t="s">
-        <v>103</v>
-      </c>
       <c r="H31" s="14" t="s">
-        <v>132</v>
+        <v>131</v>
       </c>
       <c r="I31" s="14">
         <v>612</v>
       </c>
       <c r="J31" s="14" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
       <c r="K31" s="14">
         <v>2021</v>
       </c>
       <c r="L31" s="17" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="M31" s="18"/>
       <c r="N31" s="18"/>
@@ -28923,7 +28922,7 @@
     </row>
     <row r="32" spans="1:26" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A32" s="14" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="B32" s="15">
         <v>12.63189</v>
@@ -28938,25 +28937,25 @@
         <v>9</v>
       </c>
       <c r="F32" s="14" t="s">
+        <v>132</v>
+      </c>
+      <c r="G32" s="14" t="s">
+        <v>102</v>
+      </c>
+      <c r="H32" s="14" t="s">
         <v>133</v>
-      </c>
-      <c r="G32" s="14" t="s">
-        <v>103</v>
-      </c>
-      <c r="H32" s="14" t="s">
-        <v>134</v>
       </c>
       <c r="I32" s="14">
         <v>150000</v>
       </c>
       <c r="J32" s="14" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="K32" s="14">
         <v>2021</v>
       </c>
       <c r="L32" s="17" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="M32" s="18"/>
       <c r="N32" s="18"/>
@@ -28975,7 +28974,7 @@
     </row>
     <row r="33" spans="1:26" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A33" s="14" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="B33" s="15">
         <v>11.556369999999999</v>
@@ -28990,25 +28989,25 @@
         <v>9</v>
       </c>
       <c r="F33" s="14" t="s">
-        <v>133</v>
+        <v>132</v>
       </c>
       <c r="G33" s="14" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="H33" s="14" t="s">
-        <v>135</v>
+        <v>134</v>
       </c>
       <c r="I33" s="14">
         <v>153333.33333333331</v>
       </c>
       <c r="J33" s="14" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="K33" s="14">
         <v>2021</v>
       </c>
       <c r="L33" s="17" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="M33" s="18"/>
       <c r="N33" s="18"/>
@@ -29027,7 +29026,7 @@
     </row>
     <row r="34" spans="1:26" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A34" s="14" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="B34" s="15">
         <v>12.08798</v>
@@ -29042,25 +29041,25 @@
         <v>9</v>
       </c>
       <c r="F34" s="14" t="s">
-        <v>133</v>
+        <v>132</v>
       </c>
       <c r="G34" s="14" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="H34" s="14" t="s">
-        <v>136</v>
+        <v>135</v>
       </c>
       <c r="I34" s="14">
         <v>120000</v>
       </c>
       <c r="J34" s="14" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="K34" s="14">
         <v>2021</v>
       </c>
       <c r="L34" s="17" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="M34" s="18"/>
       <c r="N34" s="18"/>
@@ -29079,7 +29078,7 @@
     </row>
     <row r="35" spans="1:26" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A35" s="14" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="B35" s="15">
         <v>11.428890000000001</v>
@@ -29094,25 +29093,25 @@
         <v>9</v>
       </c>
       <c r="F35" s="14" t="s">
+        <v>136</v>
+      </c>
+      <c r="G35" s="14" t="s">
+        <v>102</v>
+      </c>
+      <c r="H35" s="14" t="s">
         <v>137</v>
-      </c>
-      <c r="G35" s="14" t="s">
-        <v>103</v>
-      </c>
-      <c r="H35" s="14" t="s">
-        <v>138</v>
       </c>
       <c r="I35" s="14">
         <v>222000</v>
       </c>
       <c r="J35" s="14" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="K35" s="14">
         <v>2021</v>
       </c>
       <c r="L35" s="17" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="M35" s="18"/>
       <c r="N35" s="18"/>
@@ -29131,7 +29130,7 @@
     </row>
     <row r="36" spans="1:26" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A36" s="14" t="s">
-        <v>37</v>
+        <v>162</v>
       </c>
       <c r="B36" s="15">
         <v>10.943759999999999</v>
@@ -29146,25 +29145,25 @@
         <v>9</v>
       </c>
       <c r="F36" s="14" t="s">
-        <v>133</v>
+        <v>132</v>
       </c>
       <c r="G36" s="14" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="H36" s="14" t="s">
-        <v>139</v>
+        <v>138</v>
       </c>
       <c r="I36" s="14">
         <v>203125</v>
       </c>
       <c r="J36" s="14" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="K36" s="14">
         <v>2021</v>
       </c>
       <c r="L36" s="17" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="M36" s="18"/>
       <c r="N36" s="18"/>
@@ -29198,25 +29197,25 @@
         <v>9</v>
       </c>
       <c r="F37" s="14" t="s">
+        <v>139</v>
+      </c>
+      <c r="G37" s="14" t="s">
         <v>140</v>
       </c>
-      <c r="G37" s="14" t="s">
+      <c r="H37" s="14" t="s">
         <v>141</v>
-      </c>
-      <c r="H37" s="14" t="s">
-        <v>142</v>
       </c>
       <c r="I37" s="14">
         <v>195000</v>
       </c>
       <c r="J37" s="14" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="K37" s="14">
         <v>2021</v>
       </c>
       <c r="L37" s="17" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="M37" s="18"/>
       <c r="N37" s="18"/>
@@ -29250,25 +29249,25 @@
         <v>9</v>
       </c>
       <c r="F38" s="14" t="s">
+        <v>142</v>
+      </c>
+      <c r="G38" s="14" t="s">
+        <v>102</v>
+      </c>
+      <c r="H38" s="14" t="s">
         <v>143</v>
-      </c>
-      <c r="G38" s="14" t="s">
-        <v>103</v>
-      </c>
-      <c r="H38" s="14" t="s">
-        <v>144</v>
       </c>
       <c r="I38" s="14">
         <v>380000</v>
       </c>
       <c r="J38" s="14" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="K38" s="14">
         <v>2021</v>
       </c>
       <c r="L38" s="17" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="M38" s="18"/>
       <c r="N38" s="18"/>
@@ -29287,7 +29286,7 @@
     </row>
     <row r="39" spans="1:26" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A39" s="14" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
       <c r="B39" s="15">
         <v>9.7325099999999996</v>
@@ -29302,25 +29301,25 @@
         <v>9</v>
       </c>
       <c r="F39" s="14" t="s">
-        <v>140</v>
+        <v>139</v>
       </c>
       <c r="G39" s="14" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="H39" s="14" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
       <c r="I39" s="14">
         <v>120000</v>
       </c>
       <c r="J39" s="14" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="K39" s="14">
         <v>2021</v>
       </c>
       <c r="L39" s="17" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="M39" s="18"/>
       <c r="N39" s="18"/>
@@ -29341,18 +29340,18 @@
     <row r="41" spans="1:26" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
     <row r="42" spans="1:26" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A42" s="12" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
       <c r="B42" s="19" t="s">
+        <v>56</v>
+      </c>
+      <c r="C42" s="19" t="s">
         <v>57</v>
-      </c>
-      <c r="C42" s="19" t="s">
-        <v>58</v>
       </c>
     </row>
     <row r="43" spans="1:26" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A43" s="1" t="s">
-        <v>147</v>
+        <v>146</v>
       </c>
       <c r="B43" s="4">
         <v>12.053710000000001</v>
@@ -29363,7 +29362,7 @@
     </row>
     <row r="44" spans="1:26" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A44" s="1" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="B44" s="4">
         <v>11.69642</v>
@@ -29374,7 +29373,7 @@
     </row>
     <row r="45" spans="1:26" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A45" s="1" t="s">
-        <v>148</v>
+        <v>147</v>
       </c>
       <c r="B45" s="4">
         <v>10.748810000000001</v>
@@ -29385,7 +29384,7 @@
     </row>
     <row r="46" spans="1:26" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A46" s="1" t="s">
-        <v>149</v>
+        <v>148</v>
       </c>
       <c r="B46" s="4">
         <v>9.0727600000000006</v>
@@ -29407,7 +29406,7 @@
     </row>
     <row r="48" spans="1:26" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A48" s="1" t="s">
-        <v>150</v>
+        <v>149</v>
       </c>
       <c r="B48" s="4">
         <v>8.3271999999999995</v>
@@ -29418,7 +29417,7 @@
     </row>
     <row r="49" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A49" s="1" t="s">
-        <v>151</v>
+        <v>150</v>
       </c>
       <c r="B49" s="4">
         <v>8.6266800000000003</v>
@@ -29429,7 +29428,7 @@
     </row>
     <row r="50" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A50" s="1" t="s">
-        <v>152</v>
+        <v>151</v>
       </c>
       <c r="B50" s="4">
         <v>8.4164499999999993</v>
@@ -29440,7 +29439,7 @@
     </row>
     <row r="51" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A51" s="1" t="s">
-        <v>153</v>
+        <v>152</v>
       </c>
       <c r="B51" s="4">
         <v>9.1895100000000003</v>
@@ -29451,7 +29450,7 @@
     </row>
     <row r="52" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A52" s="1" t="s">
-        <v>154</v>
+        <v>153</v>
       </c>
       <c r="B52" s="4">
         <v>7.6868600000000002</v>
@@ -29462,7 +29461,7 @@
     </row>
     <row r="53" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A53" s="1" t="s">
-        <v>155</v>
+        <v>154</v>
       </c>
       <c r="B53" s="4">
         <v>8.9330499999999997</v>
@@ -29473,7 +29472,7 @@
     </row>
     <row r="54" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A54" s="1" t="s">
-        <v>156</v>
+        <v>155</v>
       </c>
       <c r="B54" s="4">
         <v>10.991619999999999</v>
@@ -29484,7 +29483,7 @@
     </row>
     <row r="55" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A55" s="1" t="s">
-        <v>157</v>
+        <v>156</v>
       </c>
       <c r="B55" s="4">
         <v>11.338749999999999</v>
@@ -29495,7 +29494,7 @@
     </row>
     <row r="56" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A56" s="1" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
       <c r="B56" s="4">
         <v>13.77692</v>
@@ -29506,7 +29505,7 @@
     </row>
     <row r="57" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A57" s="1" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="B57" s="4">
         <v>12.31551</v>
@@ -29528,19 +29527,19 @@
     </row>
     <row r="59" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
     <row r="60" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A60" s="22" t="s">
+      <c r="A60" s="21" t="s">
+        <v>158</v>
+      </c>
+      <c r="B60" s="22" t="s">
+        <v>56</v>
+      </c>
+      <c r="C60" s="22" t="s">
+        <v>57</v>
+      </c>
+    </row>
+    <row r="61" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A61" s="20" t="s">
         <v>159</v>
-      </c>
-      <c r="B60" s="23" t="s">
-        <v>57</v>
-      </c>
-      <c r="C60" s="23" t="s">
-        <v>58</v>
-      </c>
-    </row>
-    <row r="61" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A61" s="21" t="s">
-        <v>160</v>
       </c>
       <c r="B61" s="2">
         <v>12.274480000000001</v>
@@ -29551,19 +29550,19 @@
     </row>
     <row r="62" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
     <row r="63" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A63" s="23" t="s">
-        <v>161</v>
-      </c>
-      <c r="B63" s="23" t="s">
+      <c r="A63" s="22" t="s">
+        <v>160</v>
+      </c>
+      <c r="B63" s="22" t="s">
+        <v>56</v>
+      </c>
+      <c r="C63" s="22" t="s">
         <v>57</v>
-      </c>
-      <c r="C63" s="23" t="s">
-        <v>58</v>
       </c>
     </row>
     <row r="64" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A64" s="4" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="B64" s="4">
         <v>10.64</v>

</xml_diff>